<commit_message>
Fixed pannels rotation to match PCB
</commit_message>
<xml_diff>
--- a/Software/img_creator.xlsx
+++ b/Software/img_creator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\v.philippoz\Documents\pharmacy\Software\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{058E856F-EB3B-4E52-8578-1019B198EB5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D879814F-AC89-4E42-AA99-272D964640DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{77867C16-3228-4F29-99DA-0200D1AC6313}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{77867C16-3228-4F29-99DA-0200D1AC6313}"/>
   </bookViews>
   <sheets>
     <sheet name="Single pannel" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="44">
   <si>
     <t>chiffre</t>
   </si>
@@ -141,18 +141,6 @@
     <t>right</t>
   </si>
   <si>
-    <t>TopLeft</t>
-  </si>
-  <si>
-    <t>RightBottom</t>
-  </si>
-  <si>
-    <t>CenterNone</t>
-  </si>
-  <si>
-    <t>MSBLSB</t>
-  </si>
-  <si>
     <t>Binaires</t>
   </si>
   <si>
@@ -165,22 +153,25 @@
     <t>Left</t>
   </si>
   <si>
-    <t>TOP LEFT</t>
-  </si>
-  <si>
     <t>Right</t>
   </si>
   <si>
     <t>Bottom</t>
   </si>
   <si>
-    <t>RIGHT BOTTOM</t>
-  </si>
-  <si>
     <t>CENTER NONE</t>
   </si>
   <si>
     <t>Center</t>
+  </si>
+  <si>
+    <t>TOP RIGHT</t>
+  </si>
+  <si>
+    <t>LEFT BOTTOM</t>
+  </si>
+  <si>
+    <t>rotation of 90° necessary for each panel</t>
   </si>
 </sst>
 </file>
@@ -1411,10 +1402,10 @@
   <sheetData>
     <row r="1" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="AC1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="AD1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1458,18 +1449,15 @@
       <c r="W2" s="15"/>
       <c r="X2" s="15"/>
       <c r="Y2" s="17"/>
-      <c r="AA2" t="s">
-        <v>36</v>
-      </c>
       <c r="AB2" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC2" t="str">
-        <f>_xlfn.CONCAT(J2:Q2)</f>
+        <f>_xlfn.CONCAT(Q2:Q9)</f>
         <v>11111111</v>
       </c>
       <c r="AD2" t="str">
-        <f t="shared" ref="AD2:AD10" si="0">IF(BIN2DEC(AC2)&lt;16,"0","")&amp;BIN2HEX(AC2)</f>
+        <f t="shared" ref="AD2:AD9" si="0">IF(BIN2DEC(AC2)&lt;16,"0","")&amp;BIN2HEX(AC2)</f>
         <v>FF</v>
       </c>
       <c r="AF2" t="s">
@@ -1481,7 +1469,7 @@
       </c>
       <c r="AH2" s="11" t="str">
         <f>_xlfn.TEXTJOIN(", ",TRUE,AG2:AG9)</f>
-        <v>0xFFFF, 0x8180, 0x8180, 0x8180, 0x8180, 0x8180, 0x8180, 0x81FF</v>
+        <v>0xFFFF, 0x8081, 0x8081, 0x8081, 0x8081, 0x8081, 0x8081, 0xFF81</v>
       </c>
     </row>
     <row r="3" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1525,23 +1513,20 @@
       <c r="W3" s="19"/>
       <c r="X3" s="19"/>
       <c r="Y3" s="21"/>
-      <c r="AA3" t="s">
-        <v>33</v>
-      </c>
       <c r="AB3" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC3" t="str">
-        <f t="shared" ref="AC3:AC9" si="1">_xlfn.CONCAT(J3:Q3)</f>
-        <v>10000001</v>
+        <f>_xlfn.CONCAT(P2:P9)</f>
+        <v>10000000</v>
       </c>
       <c r="AD3" t="str">
         <f t="shared" si="0"/>
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AG3" t="str">
-        <f t="shared" ref="AG3:AG9" si="2">"0x"&amp;AD3&amp;AD11</f>
-        <v>0x8180</v>
+        <f t="shared" ref="AG3:AG9" si="1">"0x"&amp;AD3&amp;AD11</f>
+        <v>0x8081</v>
       </c>
     </row>
     <row r="4" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1586,19 +1571,19 @@
       <c r="X4" s="19"/>
       <c r="Y4" s="21"/>
       <c r="AB4" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC4" t="str">
-        <f t="shared" si="1"/>
-        <v>10000001</v>
+        <f>_xlfn.CONCAT(O2:O9)</f>
+        <v>10000000</v>
       </c>
       <c r="AD4" t="str">
         <f t="shared" si="0"/>
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AG4" t="str">
-        <f t="shared" si="2"/>
-        <v>0x8180</v>
+        <f t="shared" si="1"/>
+        <v>0x8081</v>
       </c>
     </row>
     <row r="5" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1642,23 +1627,20 @@
       <c r="W5" s="19"/>
       <c r="X5" s="19"/>
       <c r="Y5" s="21"/>
-      <c r="AA5" t="s">
-        <v>34</v>
-      </c>
       <c r="AB5" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC5" t="str">
-        <f t="shared" si="1"/>
-        <v>10000001</v>
+        <f>_xlfn.CONCAT(N2:N9)</f>
+        <v>10000000</v>
       </c>
       <c r="AD5" t="str">
         <f t="shared" si="0"/>
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AG5" t="str">
-        <f t="shared" si="2"/>
-        <v>0x8180</v>
+        <f t="shared" si="1"/>
+        <v>0x8081</v>
       </c>
     </row>
     <row r="6" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1703,19 +1685,19 @@
       <c r="X6" s="19"/>
       <c r="Y6" s="21"/>
       <c r="AB6" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC6" t="str">
-        <f t="shared" si="1"/>
-        <v>10000001</v>
+        <f>_xlfn.CONCAT(M2:M9)</f>
+        <v>10000000</v>
       </c>
       <c r="AD6" t="str">
         <f t="shared" si="0"/>
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AG6" t="str">
-        <f t="shared" si="2"/>
-        <v>0x8180</v>
+        <f t="shared" si="1"/>
+        <v>0x8081</v>
       </c>
     </row>
     <row r="7" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1759,23 +1741,20 @@
       <c r="W7" s="19"/>
       <c r="X7" s="19"/>
       <c r="Y7" s="21"/>
-      <c r="AA7" t="s">
+      <c r="AB7" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="AB7" s="11" t="s">
-        <v>39</v>
-      </c>
       <c r="AC7" t="str">
-        <f t="shared" si="1"/>
-        <v>10000001</v>
+        <f>_xlfn.CONCAT(L2:L9)</f>
+        <v>10000000</v>
       </c>
       <c r="AD7" t="str">
         <f t="shared" si="0"/>
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AG7" t="str">
-        <f t="shared" si="2"/>
-        <v>0x8180</v>
+        <f t="shared" si="1"/>
+        <v>0x8081</v>
       </c>
     </row>
     <row r="8" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1820,19 +1799,19 @@
       <c r="X8" s="19"/>
       <c r="Y8" s="21"/>
       <c r="AB8" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC8" t="str">
-        <f t="shared" si="1"/>
-        <v>10000001</v>
+        <f>_xlfn.CONCAT(K2:K9)</f>
+        <v>10000000</v>
       </c>
       <c r="AD8" t="str">
         <f t="shared" si="0"/>
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AG8" t="str">
-        <f t="shared" si="2"/>
-        <v>0x8180</v>
+        <f t="shared" si="1"/>
+        <v>0x8081</v>
       </c>
     </row>
     <row r="9" spans="2:34" x14ac:dyDescent="0.25">
@@ -1877,19 +1856,19 @@
       <c r="X9" s="19"/>
       <c r="Y9" s="21"/>
       <c r="AB9" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC9" t="str">
-        <f t="shared" si="1"/>
-        <v>10000001</v>
+        <f>_xlfn.CONCAT(J2:J9)</f>
+        <v>11111111</v>
       </c>
       <c r="AD9" t="str">
         <f t="shared" si="0"/>
-        <v>81</v>
+        <v>FF</v>
       </c>
       <c r="AG9" t="str">
-        <f t="shared" si="2"/>
-        <v>0x81FF</v>
+        <f t="shared" si="1"/>
+        <v>0xFF81</v>
       </c>
     </row>
     <row r="10" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1966,26 +1945,26 @@
         <v>1</v>
       </c>
       <c r="AB10" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC10" t="str">
-        <f>_xlfn.CONCAT(B10:I10)</f>
+        <f>_xlfn.CONCAT(Y10:Y17)</f>
         <v>11111111</v>
       </c>
       <c r="AD10" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(BIN2DEC(AC10)&lt;16,"0","")&amp;BIN2HEX(AC10)</f>
         <v>FF</v>
       </c>
       <c r="AF10" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="AG10" t="str">
         <f>"0x"&amp;AD18&amp;AD26</f>
-        <v>0xFF81</v>
+        <v>0x81FF</v>
       </c>
       <c r="AH10" s="12" t="str">
         <f>_xlfn.TEXTJOIN(", ",TRUE,AG10:AG17)</f>
-        <v>0xFF81, 0x0181, 0x0181, 0x0181, 0x0181, 0x0181, 0x0181, 0xFFFF</v>
+        <v>0x81FF, 0x8101, 0x8101, 0x8101, 0x8101, 0x8101, 0x8101, 0xFFFF</v>
       </c>
     </row>
     <row r="11" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2062,19 +2041,19 @@
         <v>1</v>
       </c>
       <c r="AB11" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC11" t="str">
-        <f t="shared" ref="AC11:AC17" si="3">_xlfn.CONCAT(B11:I11)</f>
-        <v>10000000</v>
+        <f>_xlfn.CONCAT(X10:X17)</f>
+        <v>10000001</v>
       </c>
       <c r="AD11" t="str">
         <f>IF(BIN2DEC(AC11)&lt;16,"0","")&amp;BIN2HEX(AC11)</f>
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="AG11" t="str">
         <f>"0x"&amp;AD19&amp;AD27</f>
-        <v>0x0181</v>
+        <v>0x8101</v>
       </c>
     </row>
     <row r="12" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2151,19 +2130,19 @@
         <v>1</v>
       </c>
       <c r="AB12" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC12" t="str">
-        <f t="shared" si="3"/>
-        <v>10000000</v>
+        <f>_xlfn.CONCAT(W10:W17)</f>
+        <v>10000001</v>
       </c>
       <c r="AD12" t="str">
-        <f t="shared" ref="AD12:AD42" si="4">IF(BIN2DEC(AC12)&lt;16,"0","")&amp;BIN2HEX(AC12)</f>
-        <v>80</v>
+        <f>IF(BIN2DEC(AC12)&lt;16,"0","")&amp;BIN2HEX(AC12)</f>
+        <v>81</v>
       </c>
       <c r="AG12" t="str">
         <f>"0x"&amp;AD20&amp;AD28</f>
-        <v>0x0181</v>
+        <v>0x8101</v>
       </c>
     </row>
     <row r="13" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2240,19 +2219,19 @@
         <v>1</v>
       </c>
       <c r="AB13" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC13" t="str">
-        <f t="shared" si="3"/>
-        <v>10000000</v>
+        <f>_xlfn.CONCAT(V10:V17)</f>
+        <v>10000001</v>
       </c>
       <c r="AD13" t="str">
-        <f t="shared" si="4"/>
-        <v>80</v>
+        <f>IF(BIN2DEC(AC13)&lt;16,"0","")&amp;BIN2HEX(AC13)</f>
+        <v>81</v>
       </c>
       <c r="AG13" t="str">
         <f>"0x"&amp;AD21&amp;AD29</f>
-        <v>0x0181</v>
+        <v>0x8101</v>
       </c>
     </row>
     <row r="14" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2329,19 +2308,19 @@
         <v>1</v>
       </c>
       <c r="AB14" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC14" t="str">
-        <f t="shared" si="3"/>
-        <v>10000000</v>
+        <f>_xlfn.CONCAT(U10:U17)</f>
+        <v>10000001</v>
       </c>
       <c r="AD14" t="str">
-        <f t="shared" si="4"/>
-        <v>80</v>
+        <f>IF(BIN2DEC(AC14)&lt;16,"0","")&amp;BIN2HEX(AC14)</f>
+        <v>81</v>
       </c>
       <c r="AG14" t="str">
         <f>"0x"&amp;AD22&amp;AD30</f>
-        <v>0x0181</v>
+        <v>0x8101</v>
       </c>
     </row>
     <row r="15" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2418,19 +2397,19 @@
         <v>1</v>
       </c>
       <c r="AB15" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC15" t="str">
-        <f t="shared" si="3"/>
-        <v>10000000</v>
+        <f>_xlfn.CONCAT(T10:T17)</f>
+        <v>10000001</v>
       </c>
       <c r="AD15" t="str">
-        <f t="shared" si="4"/>
-        <v>80</v>
+        <f>IF(BIN2DEC(AC15)&lt;16,"0","")&amp;BIN2HEX(AC15)</f>
+        <v>81</v>
       </c>
       <c r="AG15" t="str">
         <f>"0x"&amp;AD23&amp;AD31</f>
-        <v>0x0181</v>
+        <v>0x8101</v>
       </c>
     </row>
     <row r="16" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2507,19 +2486,19 @@
         <v>1</v>
       </c>
       <c r="AB16" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC16" t="str">
-        <f t="shared" si="3"/>
-        <v>10000000</v>
+        <f>_xlfn.CONCAT(S10:S17)</f>
+        <v>10000001</v>
       </c>
       <c r="AD16" t="str">
-        <f t="shared" si="4"/>
-        <v>80</v>
+        <f>IF(BIN2DEC(AC16)&lt;16,"0","")&amp;BIN2HEX(AC16)</f>
+        <v>81</v>
       </c>
       <c r="AG16" t="str">
         <f>"0x"&amp;AD24&amp;AD32</f>
-        <v>0x0181</v>
+        <v>0x8101</v>
       </c>
     </row>
     <row r="17" spans="2:34" x14ac:dyDescent="0.25">
@@ -2596,15 +2575,15 @@
         <v>1</v>
       </c>
       <c r="AB17" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC17" t="str">
-        <f t="shared" si="3"/>
-        <v>11111111</v>
+        <f>_xlfn.CONCAT(R10:R17)</f>
+        <v>10000001</v>
       </c>
       <c r="AD17" t="str">
-        <f t="shared" si="4"/>
-        <v>FF</v>
+        <f>IF(BIN2DEC(AC17)&lt;16,"0","")&amp;BIN2HEX(AC17)</f>
+        <v>81</v>
       </c>
       <c r="AG17" t="str">
         <f>"0x"&amp;AD25&amp;AD33</f>
@@ -2653,25 +2632,25 @@
       <c r="X18" s="19"/>
       <c r="Y18" s="21"/>
       <c r="AB18" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC18" t="str">
-        <f>_xlfn.CONCAT(R10:Y10)</f>
-        <v>11111111</v>
+        <f>_xlfn.CONCAT(I10:I17)</f>
+        <v>10000001</v>
       </c>
       <c r="AD18" t="str">
-        <f t="shared" si="4"/>
-        <v>FF</v>
+        <f>IF(BIN2DEC(AC18)&lt;16,"0","")&amp;BIN2HEX(AC18)</f>
+        <v>81</v>
       </c>
       <c r="AF18" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="AG18" t="str">
         <f>"0x"&amp;AD34&amp;"00"</f>
         <v>0x8100</v>
       </c>
       <c r="AH18" s="10" t="str">
-        <f t="shared" ref="AH18" si="5">_xlfn.TEXTJOIN(", ",TRUE,AG18:AG25)</f>
+        <f t="shared" ref="AH18" si="2">_xlfn.TEXTJOIN(", ",TRUE,AG18:AG25)</f>
         <v>0x8100, 0x0000, 0x0000, 0x0000, 0x0000, 0x0000, 0x0000, 0x8100</v>
       </c>
     </row>
@@ -2717,18 +2696,18 @@
       <c r="X19" s="19"/>
       <c r="Y19" s="21"/>
       <c r="AB19" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC19" t="str">
-        <f t="shared" ref="AC19:AC25" si="6">_xlfn.CONCAT(R11:Y11)</f>
-        <v>00000001</v>
+        <f>_xlfn.CONCAT(H10:H17)</f>
+        <v>10000001</v>
       </c>
       <c r="AD19" t="str">
-        <f t="shared" si="4"/>
-        <v>01</v>
+        <f>IF(BIN2DEC(AC19)&lt;16,"0","")&amp;BIN2HEX(AC19)</f>
+        <v>81</v>
       </c>
       <c r="AG19" t="str">
-        <f t="shared" ref="AG19:AG25" si="7">"0x"&amp;AD35&amp;"00"</f>
+        <f t="shared" ref="AG19:AG25" si="3">"0x"&amp;AD35&amp;"00"</f>
         <v>0x0000</v>
       </c>
     </row>
@@ -2774,18 +2753,18 @@
       <c r="X20" s="19"/>
       <c r="Y20" s="21"/>
       <c r="AB20" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC20" t="str">
-        <f t="shared" si="6"/>
-        <v>00000001</v>
+        <f>_xlfn.CONCAT(G10:G17)</f>
+        <v>10000001</v>
       </c>
       <c r="AD20" t="str">
-        <f t="shared" si="4"/>
-        <v>01</v>
+        <f>IF(BIN2DEC(AC20)&lt;16,"0","")&amp;BIN2HEX(AC20)</f>
+        <v>81</v>
       </c>
       <c r="AG20" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>0x0000</v>
       </c>
     </row>
@@ -2831,18 +2810,18 @@
       <c r="X21" s="19"/>
       <c r="Y21" s="21"/>
       <c r="AB21" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC21" t="str">
-        <f t="shared" si="6"/>
-        <v>00000001</v>
+        <f>_xlfn.CONCAT(F10:F17)</f>
+        <v>10000001</v>
       </c>
       <c r="AD21" t="str">
-        <f t="shared" si="4"/>
-        <v>01</v>
+        <f>IF(BIN2DEC(AC21)&lt;16,"0","")&amp;BIN2HEX(AC21)</f>
+        <v>81</v>
       </c>
       <c r="AG21" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>0x0000</v>
       </c>
     </row>
@@ -2888,18 +2867,18 @@
       <c r="X22" s="19"/>
       <c r="Y22" s="21"/>
       <c r="AB22" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC22" t="str">
-        <f t="shared" si="6"/>
-        <v>00000001</v>
+        <f>_xlfn.CONCAT(E10:E17)</f>
+        <v>10000001</v>
       </c>
       <c r="AD22" t="str">
-        <f t="shared" si="4"/>
-        <v>01</v>
+        <f>IF(BIN2DEC(AC22)&lt;16,"0","")&amp;BIN2HEX(AC22)</f>
+        <v>81</v>
       </c>
       <c r="AG22" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>0x0000</v>
       </c>
     </row>
@@ -2945,18 +2924,18 @@
       <c r="X23" s="19"/>
       <c r="Y23" s="21"/>
       <c r="AB23" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC23" t="str">
-        <f t="shared" si="6"/>
-        <v>00000001</v>
+        <f>_xlfn.CONCAT(D10:D17)</f>
+        <v>10000001</v>
       </c>
       <c r="AD23" t="str">
-        <f t="shared" si="4"/>
-        <v>01</v>
+        <f>IF(BIN2DEC(AC23)&lt;16,"0","")&amp;BIN2HEX(AC23)</f>
+        <v>81</v>
       </c>
       <c r="AG23" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>0x0000</v>
       </c>
     </row>
@@ -3002,18 +2981,18 @@
       <c r="X24" s="19"/>
       <c r="Y24" s="21"/>
       <c r="AB24" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC24" t="str">
-        <f t="shared" si="6"/>
-        <v>00000001</v>
+        <f>_xlfn.CONCAT(C10:C17)</f>
+        <v>10000001</v>
       </c>
       <c r="AD24" t="str">
-        <f t="shared" si="4"/>
-        <v>01</v>
+        <f>IF(BIN2DEC(AC24)&lt;16,"0","")&amp;BIN2HEX(AC24)</f>
+        <v>81</v>
       </c>
       <c r="AG24" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>0x0000</v>
       </c>
     </row>
@@ -3059,32 +3038,32 @@
       <c r="X25" s="25"/>
       <c r="Y25" s="27"/>
       <c r="AB25" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC25" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.CONCAT(B10:B17)</f>
         <v>11111111</v>
       </c>
       <c r="AD25" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(BIN2DEC(AC25)&lt;16,"0","")&amp;BIN2HEX(AC25)</f>
         <v>FF</v>
       </c>
       <c r="AG25" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>0x8100</v>
       </c>
     </row>
     <row r="26" spans="2:34" x14ac:dyDescent="0.25">
       <c r="AB26" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC26" t="str">
-        <f>_xlfn.CONCAT(J18:Q18)</f>
-        <v>10000001</v>
+        <f>_xlfn.CONCAT(Q18:Q25)</f>
+        <v>11111111</v>
       </c>
       <c r="AD26" t="str">
-        <f t="shared" si="4"/>
-        <v>81</v>
+        <f t="shared" ref="AD26:AD41" si="4">IF(BIN2DEC(AC26)&lt;16,"0","")&amp;BIN2HEX(AC26)</f>
+        <v>FF</v>
       </c>
       <c r="AH26" s="13"/>
     </row>
@@ -3093,37 +3072,40 @@
         <v>28</v>
       </c>
       <c r="AB27" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC27" t="str">
-        <f t="shared" ref="AC27:AC33" si="8">_xlfn.CONCAT(J19:Q19)</f>
-        <v>10000001</v>
+        <f>_xlfn.CONCAT(P18:P25)</f>
+        <v>00000001</v>
       </c>
       <c r="AD27" t="str">
         <f t="shared" si="4"/>
-        <v>81</v>
+        <v>01</v>
       </c>
     </row>
     <row r="28" spans="2:34" x14ac:dyDescent="0.25">
-      <c r="L28" s="11" t="s">
+      <c r="L28" s="12" t="s">
         <v>31</v>
       </c>
       <c r="M28" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="O28" s="9" t="s">
+      <c r="O28" s="11" t="s">
         <v>32</v>
       </c>
+      <c r="Q28" t="s">
+        <v>43</v>
+      </c>
       <c r="AB28" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC28" t="str">
-        <f t="shared" si="8"/>
-        <v>10000001</v>
+        <f>_xlfn.CONCAT(O18:O25)</f>
+        <v>00000001</v>
       </c>
       <c r="AD28" t="str">
         <f t="shared" si="4"/>
-        <v>81</v>
+        <v>01</v>
       </c>
     </row>
     <row r="29" spans="2:34" x14ac:dyDescent="0.25">
@@ -3131,62 +3113,62 @@
         <v>30</v>
       </c>
       <c r="AB29" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC29" t="str">
-        <f t="shared" si="8"/>
-        <v>10000001</v>
+        <f>_xlfn.CONCAT(N18:N25)</f>
+        <v>00000001</v>
       </c>
       <c r="AD29" t="str">
         <f t="shared" si="4"/>
-        <v>81</v>
+        <v>01</v>
       </c>
     </row>
     <row r="30" spans="2:34" x14ac:dyDescent="0.25">
       <c r="AB30" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC30" t="str">
-        <f t="shared" si="8"/>
-        <v>10000001</v>
+        <f>_xlfn.CONCAT(M18:M25)</f>
+        <v>00000001</v>
       </c>
       <c r="AD30" t="str">
         <f t="shared" si="4"/>
-        <v>81</v>
+        <v>01</v>
       </c>
     </row>
     <row r="31" spans="2:34" x14ac:dyDescent="0.25">
       <c r="AB31" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC31" t="str">
-        <f t="shared" si="8"/>
-        <v>10000001</v>
+        <f>_xlfn.CONCAT(L18:L25)</f>
+        <v>00000001</v>
       </c>
       <c r="AD31" t="str">
         <f t="shared" si="4"/>
-        <v>81</v>
+        <v>01</v>
       </c>
     </row>
     <row r="32" spans="2:34" x14ac:dyDescent="0.25">
       <c r="AB32" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC32" t="str">
-        <f t="shared" si="8"/>
-        <v>10000001</v>
+        <f>_xlfn.CONCAT(K18:K25)</f>
+        <v>00000001</v>
       </c>
       <c r="AD32" t="str">
         <f t="shared" si="4"/>
-        <v>81</v>
+        <v>01</v>
       </c>
     </row>
     <row r="33" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB33" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC33" t="str">
-        <f t="shared" si="8"/>
+        <f>_xlfn.CONCAT(J18:J25)</f>
         <v>11111111</v>
       </c>
       <c r="AD33" t="str">
@@ -3196,10 +3178,10 @@
     </row>
     <row r="34" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB34" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC34" t="str">
-        <f>_xlfn.CONCAT(J10:Q10)</f>
+        <f>_xlfn.CONCAT(Q10:Q17)</f>
         <v>10000001</v>
       </c>
       <c r="AD34" t="str">
@@ -3209,10 +3191,10 @@
     </row>
     <row r="35" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB35" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC35" t="str">
-        <f t="shared" ref="AC35:AC42" si="9">_xlfn.CONCAT(J11:Q11)</f>
+        <f>_xlfn.CONCAT(P10:P17)</f>
         <v>00000000</v>
       </c>
       <c r="AD35" t="str">
@@ -3222,10 +3204,10 @@
     </row>
     <row r="36" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB36" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC36" t="str">
-        <f t="shared" si="9"/>
+        <f>_xlfn.CONCAT(O10:O17)</f>
         <v>00000000</v>
       </c>
       <c r="AD36" t="str">
@@ -3235,10 +3217,10 @@
     </row>
     <row r="37" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB37" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC37" t="str">
-        <f t="shared" si="9"/>
+        <f>_xlfn.CONCAT(N10:N17)</f>
         <v>00000000</v>
       </c>
       <c r="AD37" t="str">
@@ -3248,10 +3230,10 @@
     </row>
     <row r="38" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB38" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC38" t="str">
-        <f t="shared" si="9"/>
+        <f>_xlfn.CONCAT(M9:M16)</f>
         <v>00000000</v>
       </c>
       <c r="AD38" t="str">
@@ -3261,10 +3243,10 @@
     </row>
     <row r="39" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB39" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC39" t="str">
-        <f t="shared" si="9"/>
+        <f>_xlfn.CONCAT(L10:L17)</f>
         <v>00000000</v>
       </c>
       <c r="AD39" t="str">
@@ -3274,10 +3256,10 @@
     </row>
     <row r="40" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB40" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC40" t="str">
-        <f t="shared" si="9"/>
+        <f>_xlfn.CONCAT(K10:K17)</f>
         <v>00000000</v>
       </c>
       <c r="AD40" t="str">
@@ -3287,10 +3269,10 @@
     </row>
     <row r="41" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB41" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC41" t="str">
-        <f t="shared" si="9"/>
+        <f>_xlfn.CONCAT(J10:J17)</f>
         <v>10000001</v>
       </c>
       <c r="AD41" t="str">
@@ -3337,10 +3319,10 @@
   <sheetData>
     <row r="1" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="AC1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="AD1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3384,14 +3366,11 @@
       <c r="W2" s="15"/>
       <c r="X2" s="15"/>
       <c r="Y2" s="17"/>
-      <c r="AA2" t="s">
-        <v>36</v>
-      </c>
       <c r="AB2" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC2" t="str">
-        <f>_xlfn.CONCAT(J2:Q2)</f>
+        <f>_xlfn.CONCAT(Q2:Q9)</f>
         <v>00000000</v>
       </c>
       <c r="AD2" t="str">
@@ -3407,7 +3386,7 @@
       </c>
       <c r="AH2" s="11" t="str">
         <f>_xlfn.TEXTJOIN(", ",TRUE,AG2:AG9)</f>
-        <v>0x0000, 0x7E7F, 0x4240, 0x4240, 0x4240, 0x4240, 0x427F, 0x4200</v>
+        <v>0x0000, 0x7F7E, 0x4042, 0x4042, 0x4042, 0x4042, 0x7F42, 0x0042</v>
       </c>
     </row>
     <row r="3" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3451,23 +3430,20 @@
       <c r="W3" s="19"/>
       <c r="X3" s="19"/>
       <c r="Y3" s="21"/>
-      <c r="AA3" t="s">
-        <v>33</v>
-      </c>
       <c r="AB3" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC3" t="str">
-        <f t="shared" ref="AC3:AC9" si="1">_xlfn.CONCAT(J3:Q3)</f>
-        <v>01111110</v>
+        <f>_xlfn.CONCAT(P2:P9)</f>
+        <v>01111111</v>
       </c>
       <c r="AD3" t="str">
         <f t="shared" si="0"/>
-        <v>7E</v>
+        <v>7F</v>
       </c>
       <c r="AG3" t="str">
-        <f t="shared" ref="AG3:AG9" si="2">"0x"&amp;AD3&amp;AD11</f>
-        <v>0x7E7F</v>
+        <f t="shared" ref="AG3:AG9" si="1">"0x"&amp;AD3&amp;AD11</f>
+        <v>0x7F7E</v>
       </c>
     </row>
     <row r="4" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3512,19 +3488,19 @@
       <c r="X4" s="19"/>
       <c r="Y4" s="21"/>
       <c r="AB4" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC4" t="str">
-        <f t="shared" si="1"/>
-        <v>01000010</v>
+        <f>_xlfn.CONCAT(O2:O9)</f>
+        <v>01000000</v>
       </c>
       <c r="AD4" t="str">
         <f t="shared" si="0"/>
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="AG4" t="str">
-        <f t="shared" si="2"/>
-        <v>0x4240</v>
+        <f t="shared" si="1"/>
+        <v>0x4042</v>
       </c>
     </row>
     <row r="5" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3568,23 +3544,20 @@
       <c r="W5" s="19"/>
       <c r="X5" s="19"/>
       <c r="Y5" s="21"/>
-      <c r="AA5" t="s">
-        <v>34</v>
-      </c>
       <c r="AB5" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC5" t="str">
-        <f t="shared" si="1"/>
-        <v>01000010</v>
+        <f>_xlfn.CONCAT(N2:N9)</f>
+        <v>01000000</v>
       </c>
       <c r="AD5" t="str">
         <f t="shared" si="0"/>
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="AG5" t="str">
-        <f t="shared" si="2"/>
-        <v>0x4240</v>
+        <f t="shared" si="1"/>
+        <v>0x4042</v>
       </c>
     </row>
     <row r="6" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3629,19 +3602,19 @@
       <c r="X6" s="19"/>
       <c r="Y6" s="21"/>
       <c r="AB6" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC6" t="str">
-        <f t="shared" si="1"/>
-        <v>01000010</v>
+        <f>_xlfn.CONCAT(M2:M9)</f>
+        <v>01000000</v>
       </c>
       <c r="AD6" t="str">
         <f t="shared" si="0"/>
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="AG6" t="str">
-        <f t="shared" si="2"/>
-        <v>0x4240</v>
+        <f t="shared" si="1"/>
+        <v>0x4042</v>
       </c>
     </row>
     <row r="7" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3685,23 +3658,20 @@
       <c r="W7" s="19"/>
       <c r="X7" s="19"/>
       <c r="Y7" s="21"/>
-      <c r="AA7" t="s">
+      <c r="AB7" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="AB7" s="11" t="s">
-        <v>39</v>
-      </c>
       <c r="AC7" t="str">
-        <f t="shared" si="1"/>
-        <v>01000010</v>
+        <f>_xlfn.CONCAT(L2:L9)</f>
+        <v>01000000</v>
       </c>
       <c r="AD7" t="str">
         <f t="shared" si="0"/>
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="AG7" t="str">
-        <f t="shared" si="2"/>
-        <v>0x4240</v>
+        <f t="shared" si="1"/>
+        <v>0x4042</v>
       </c>
     </row>
     <row r="8" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3746,19 +3716,19 @@
       <c r="X8" s="19"/>
       <c r="Y8" s="21"/>
       <c r="AB8" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC8" t="str">
-        <f t="shared" si="1"/>
-        <v>01000010</v>
+        <f>_xlfn.CONCAT(K2:K9)</f>
+        <v>01111111</v>
       </c>
       <c r="AD8" t="str">
         <f t="shared" si="0"/>
-        <v>42</v>
+        <v>7F</v>
       </c>
       <c r="AG8" t="str">
-        <f t="shared" si="2"/>
-        <v>0x427F</v>
+        <f t="shared" si="1"/>
+        <v>0x7F42</v>
       </c>
     </row>
     <row r="9" spans="2:34" x14ac:dyDescent="0.25">
@@ -3803,19 +3773,19 @@
       <c r="X9" s="19"/>
       <c r="Y9" s="21"/>
       <c r="AB9" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC9" t="str">
-        <f t="shared" si="1"/>
-        <v>01000010</v>
+        <f>_xlfn.CONCAT(J2:J9)</f>
+        <v>00000000</v>
       </c>
       <c r="AD9" t="str">
         <f t="shared" si="0"/>
-        <v>42</v>
+        <v>00</v>
       </c>
       <c r="AG9" t="str">
-        <f t="shared" si="2"/>
-        <v>0x4200</v>
+        <f t="shared" si="1"/>
+        <v>0x0042</v>
       </c>
     </row>
     <row r="10" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3892,26 +3862,26 @@
         <v>0</v>
       </c>
       <c r="AB10" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC10" t="str">
-        <f>_xlfn.CONCAT(B10:I10)</f>
+        <f>_xlfn.CONCAT(Y10:Y17)</f>
         <v>00000000</v>
       </c>
       <c r="AD10" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(BIN2DEC(AC10)&lt;16,"0","")&amp;BIN2HEX(AC10)</f>
         <v>00</v>
       </c>
       <c r="AF10" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="AG10" t="str">
         <f>"0x"&amp;AD18&amp;AD26</f>
-        <v>0x0042</v>
+        <v>0x4200</v>
       </c>
       <c r="AH10" s="12" t="str">
         <f>_xlfn.TEXTJOIN(", ",TRUE,AG10:AG17)</f>
-        <v>0x0042, 0xFE42, 0x0242, 0x0242, 0x0242, 0x0242, 0xFE7E, 0x0000</v>
+        <v>0x4200, 0x42FE, 0x4202, 0x4202, 0x4202, 0x4202, 0x7EFE, 0x0000</v>
       </c>
     </row>
     <row r="11" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3988,19 +3958,19 @@
         <v>0</v>
       </c>
       <c r="AB11" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC11" t="str">
-        <f t="shared" ref="AC11:AC17" si="3">_xlfn.CONCAT(B11:I11)</f>
-        <v>01111111</v>
+        <f>_xlfn.CONCAT(X10:X17)</f>
+        <v>01111110</v>
       </c>
       <c r="AD11" t="str">
         <f>IF(BIN2DEC(AC11)&lt;16,"0","")&amp;BIN2HEX(AC11)</f>
-        <v>7F</v>
+        <v>7E</v>
       </c>
       <c r="AG11" t="str">
-        <f>"0x"&amp;AD19&amp;AD27</f>
-        <v>0xFE42</v>
+        <f t="shared" ref="AG11:AG17" si="2">"0x"&amp;AD19&amp;AD27</f>
+        <v>0x42FE</v>
       </c>
     </row>
     <row r="12" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4077,19 +4047,19 @@
         <v>0</v>
       </c>
       <c r="AB12" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC12" t="str">
-        <f t="shared" si="3"/>
-        <v>01000000</v>
+        <f>_xlfn.CONCAT(W10:W17)</f>
+        <v>01000010</v>
       </c>
       <c r="AD12" t="str">
-        <f t="shared" ref="AD12:AD41" si="4">IF(BIN2DEC(AC12)&lt;16,"0","")&amp;BIN2HEX(AC12)</f>
-        <v>40</v>
+        <f>IF(BIN2DEC(AC12)&lt;16,"0","")&amp;BIN2HEX(AC12)</f>
+        <v>42</v>
       </c>
       <c r="AG12" t="str">
-        <f>"0x"&amp;AD20&amp;AD28</f>
-        <v>0x0242</v>
+        <f t="shared" si="2"/>
+        <v>0x4202</v>
       </c>
     </row>
     <row r="13" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4166,19 +4136,19 @@
         <v>0</v>
       </c>
       <c r="AB13" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC13" t="str">
-        <f t="shared" si="3"/>
-        <v>01000000</v>
+        <f>_xlfn.CONCAT(V10:V17)</f>
+        <v>01000010</v>
       </c>
       <c r="AD13" t="str">
-        <f t="shared" si="4"/>
-        <v>40</v>
+        <f>IF(BIN2DEC(AC13)&lt;16,"0","")&amp;BIN2HEX(AC13)</f>
+        <v>42</v>
       </c>
       <c r="AG13" t="str">
-        <f>"0x"&amp;AD21&amp;AD29</f>
-        <v>0x0242</v>
+        <f t="shared" si="2"/>
+        <v>0x4202</v>
       </c>
     </row>
     <row r="14" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4255,19 +4225,19 @@
         <v>0</v>
       </c>
       <c r="AB14" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC14" t="str">
-        <f t="shared" si="3"/>
-        <v>01000000</v>
+        <f>_xlfn.CONCAT(U10:U17)</f>
+        <v>01000010</v>
       </c>
       <c r="AD14" t="str">
-        <f t="shared" si="4"/>
-        <v>40</v>
+        <f>IF(BIN2DEC(AC14)&lt;16,"0","")&amp;BIN2HEX(AC14)</f>
+        <v>42</v>
       </c>
       <c r="AG14" t="str">
-        <f>"0x"&amp;AD22&amp;AD30</f>
-        <v>0x0242</v>
+        <f t="shared" si="2"/>
+        <v>0x4202</v>
       </c>
     </row>
     <row r="15" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4344,19 +4314,19 @@
         <v>0</v>
       </c>
       <c r="AB15" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC15" t="str">
-        <f t="shared" si="3"/>
-        <v>01000000</v>
+        <f>_xlfn.CONCAT(T10:T17)</f>
+        <v>01000010</v>
       </c>
       <c r="AD15" t="str">
-        <f t="shared" si="4"/>
-        <v>40</v>
+        <f>IF(BIN2DEC(AC15)&lt;16,"0","")&amp;BIN2HEX(AC15)</f>
+        <v>42</v>
       </c>
       <c r="AG15" t="str">
-        <f>"0x"&amp;AD23&amp;AD31</f>
-        <v>0x0242</v>
+        <f t="shared" si="2"/>
+        <v>0x4202</v>
       </c>
     </row>
     <row r="16" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4433,19 +4403,19 @@
         <v>0</v>
       </c>
       <c r="AB16" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC16" t="str">
-        <f t="shared" si="3"/>
-        <v>01111111</v>
+        <f>_xlfn.CONCAT(S10:S17)</f>
+        <v>01000010</v>
       </c>
       <c r="AD16" t="str">
-        <f t="shared" si="4"/>
-        <v>7F</v>
+        <f>IF(BIN2DEC(AC16)&lt;16,"0","")&amp;BIN2HEX(AC16)</f>
+        <v>42</v>
       </c>
       <c r="AG16" t="str">
-        <f>"0x"&amp;AD24&amp;AD32</f>
-        <v>0xFE7E</v>
+        <f t="shared" si="2"/>
+        <v>0x7EFE</v>
       </c>
     </row>
     <row r="17" spans="2:34" x14ac:dyDescent="0.25">
@@ -4522,18 +4492,18 @@
         <v>0</v>
       </c>
       <c r="AB17" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC17" t="str">
-        <f t="shared" si="3"/>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(R10:R17)</f>
+        <v>01000010</v>
       </c>
       <c r="AD17" t="str">
-        <f t="shared" si="4"/>
-        <v>00</v>
+        <f>IF(BIN2DEC(AC17)&lt;16,"0","")&amp;BIN2HEX(AC17)</f>
+        <v>42</v>
       </c>
       <c r="AG17" t="str">
-        <f>"0x"&amp;AD25&amp;AD33</f>
+        <f t="shared" si="2"/>
         <v>0x0000</v>
       </c>
     </row>
@@ -4579,25 +4549,25 @@
       <c r="X18" s="19"/>
       <c r="Y18" s="21"/>
       <c r="AB18" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC18" t="str">
+        <f>_xlfn.CONCAT(I10:I17)</f>
+        <v>01000010</v>
+      </c>
+      <c r="AD18" t="str">
+        <f>IF(BIN2DEC(AC18)&lt;16,"0","")&amp;BIN2HEX(AC18)</f>
         <v>42</v>
       </c>
-      <c r="AC18" t="str">
-        <f>_xlfn.CONCAT(R10:Y10)</f>
-        <v>00000000</v>
-      </c>
-      <c r="AD18" t="str">
-        <f t="shared" si="4"/>
-        <v>00</v>
-      </c>
       <c r="AF18" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="AG18" t="str">
         <f>"0x"&amp;AD34&amp;"00"</f>
         <v>0x4200</v>
       </c>
       <c r="AH18" s="10" t="str">
-        <f t="shared" ref="AH18" si="5">_xlfn.TEXTJOIN(", ",TRUE,AG18:AG25)</f>
+        <f t="shared" ref="AH18" si="3">_xlfn.TEXTJOIN(", ",TRUE,AG18:AG25)</f>
         <v>0x4200, 0xC300, 0x0000, 0x0000, 0x0000, 0x0000, 0xC300, 0x4200</v>
       </c>
     </row>
@@ -4643,18 +4613,18 @@
       <c r="X19" s="19"/>
       <c r="Y19" s="21"/>
       <c r="AB19" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC19" t="str">
+        <f>_xlfn.CONCAT(H10:H17)</f>
+        <v>01000010</v>
+      </c>
+      <c r="AD19" t="str">
+        <f>IF(BIN2DEC(AC19)&lt;16,"0","")&amp;BIN2HEX(AC19)</f>
         <v>42</v>
       </c>
-      <c r="AC19" t="str">
-        <f t="shared" ref="AC19:AC25" si="6">_xlfn.CONCAT(R11:Y11)</f>
-        <v>11111110</v>
-      </c>
-      <c r="AD19" t="str">
-        <f t="shared" si="4"/>
-        <v>FE</v>
-      </c>
       <c r="AG19" t="str">
-        <f t="shared" ref="AG19:AG25" si="7">"0x"&amp;AD35&amp;"00"</f>
+        <f t="shared" ref="AG19:AG25" si="4">"0x"&amp;AD35&amp;"00"</f>
         <v>0xC300</v>
       </c>
     </row>
@@ -4700,18 +4670,18 @@
       <c r="X20" s="19"/>
       <c r="Y20" s="21"/>
       <c r="AB20" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC20" t="str">
+        <f>_xlfn.CONCAT(G10:G17)</f>
+        <v>01000010</v>
+      </c>
+      <c r="AD20" t="str">
+        <f>IF(BIN2DEC(AC20)&lt;16,"0","")&amp;BIN2HEX(AC20)</f>
         <v>42</v>
       </c>
-      <c r="AC20" t="str">
-        <f t="shared" si="6"/>
-        <v>00000010</v>
-      </c>
-      <c r="AD20" t="str">
+      <c r="AG20" t="str">
         <f t="shared" si="4"/>
-        <v>02</v>
-      </c>
-      <c r="AG20" t="str">
-        <f t="shared" si="7"/>
         <v>0x0000</v>
       </c>
     </row>
@@ -4757,18 +4727,18 @@
       <c r="X21" s="19"/>
       <c r="Y21" s="21"/>
       <c r="AB21" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC21" t="str">
+        <f>_xlfn.CONCAT(F10:F17)</f>
+        <v>01000010</v>
+      </c>
+      <c r="AD21" t="str">
+        <f>IF(BIN2DEC(AC21)&lt;16,"0","")&amp;BIN2HEX(AC21)</f>
         <v>42</v>
       </c>
-      <c r="AC21" t="str">
-        <f t="shared" si="6"/>
-        <v>00000010</v>
-      </c>
-      <c r="AD21" t="str">
+      <c r="AG21" t="str">
         <f t="shared" si="4"/>
-        <v>02</v>
-      </c>
-      <c r="AG21" t="str">
-        <f t="shared" si="7"/>
         <v>0x0000</v>
       </c>
     </row>
@@ -4814,18 +4784,18 @@
       <c r="X22" s="19"/>
       <c r="Y22" s="21"/>
       <c r="AB22" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC22" t="str">
+        <f>_xlfn.CONCAT(E10:E17)</f>
+        <v>01000010</v>
+      </c>
+      <c r="AD22" t="str">
+        <f>IF(BIN2DEC(AC22)&lt;16,"0","")&amp;BIN2HEX(AC22)</f>
         <v>42</v>
       </c>
-      <c r="AC22" t="str">
-        <f t="shared" si="6"/>
-        <v>00000010</v>
-      </c>
-      <c r="AD22" t="str">
+      <c r="AG22" t="str">
         <f t="shared" si="4"/>
-        <v>02</v>
-      </c>
-      <c r="AG22" t="str">
-        <f t="shared" si="7"/>
         <v>0x0000</v>
       </c>
     </row>
@@ -4871,18 +4841,18 @@
       <c r="X23" s="19"/>
       <c r="Y23" s="21"/>
       <c r="AB23" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC23" t="str">
+        <f>_xlfn.CONCAT(D10:D17)</f>
+        <v>01000010</v>
+      </c>
+      <c r="AD23" t="str">
+        <f>IF(BIN2DEC(AC23)&lt;16,"0","")&amp;BIN2HEX(AC23)</f>
         <v>42</v>
       </c>
-      <c r="AC23" t="str">
-        <f t="shared" si="6"/>
-        <v>00000010</v>
-      </c>
-      <c r="AD23" t="str">
+      <c r="AG23" t="str">
         <f t="shared" si="4"/>
-        <v>02</v>
-      </c>
-      <c r="AG23" t="str">
-        <f t="shared" si="7"/>
         <v>0x0000</v>
       </c>
     </row>
@@ -4928,18 +4898,18 @@
       <c r="X24" s="19"/>
       <c r="Y24" s="21"/>
       <c r="AB24" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC24" t="str">
-        <f t="shared" si="6"/>
-        <v>11111110</v>
+        <f>_xlfn.CONCAT(C10:C17)</f>
+        <v>01111110</v>
       </c>
       <c r="AD24" t="str">
+        <f>IF(BIN2DEC(AC24)&lt;16,"0","")&amp;BIN2HEX(AC24)</f>
+        <v>7E</v>
+      </c>
+      <c r="AG24" t="str">
         <f t="shared" si="4"/>
-        <v>FE</v>
-      </c>
-      <c r="AG24" t="str">
-        <f t="shared" si="7"/>
         <v>0xC300</v>
       </c>
     </row>
@@ -4985,32 +4955,32 @@
       <c r="X25" s="25"/>
       <c r="Y25" s="27"/>
       <c r="AB25" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC25" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.CONCAT(B10:B17)</f>
         <v>00000000</v>
       </c>
       <c r="AD25" t="str">
+        <f>IF(BIN2DEC(AC25)&lt;16,"0","")&amp;BIN2HEX(AC25)</f>
+        <v>00</v>
+      </c>
+      <c r="AG25" t="str">
         <f t="shared" si="4"/>
-        <v>00</v>
-      </c>
-      <c r="AG25" t="str">
-        <f t="shared" si="7"/>
         <v>0x4200</v>
       </c>
     </row>
     <row r="26" spans="2:34" x14ac:dyDescent="0.25">
       <c r="AB26" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC26" t="str">
-        <f>_xlfn.CONCAT(J18:Q18)</f>
-        <v>01000010</v>
+        <f>_xlfn.CONCAT(Q18:Q25)</f>
+        <v>00000000</v>
       </c>
       <c r="AD26" t="str">
-        <f t="shared" si="4"/>
-        <v>42</v>
+        <f t="shared" ref="AD12:AD41" si="5">IF(BIN2DEC(AC26)&lt;16,"0","")&amp;BIN2HEX(AC26)</f>
+        <v>00</v>
       </c>
       <c r="AH26" s="13"/>
     </row>
@@ -5019,37 +4989,40 @@
         <v>28</v>
       </c>
       <c r="AB27" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC27" t="str">
-        <f t="shared" ref="AC27:AC33" si="8">_xlfn.CONCAT(J19:Q19)</f>
-        <v>01000010</v>
+        <f>_xlfn.CONCAT(P18:P25)</f>
+        <v>11111110</v>
       </c>
       <c r="AD27" t="str">
-        <f t="shared" si="4"/>
-        <v>42</v>
+        <f t="shared" si="5"/>
+        <v>FE</v>
       </c>
     </row>
     <row r="28" spans="2:34" x14ac:dyDescent="0.25">
-      <c r="L28" s="11" t="s">
+      <c r="L28" s="12" t="s">
         <v>31</v>
       </c>
       <c r="M28" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="O28" s="9" t="s">
+      <c r="O28" s="11" t="s">
         <v>32</v>
       </c>
+      <c r="Q28" t="s">
+        <v>43</v>
+      </c>
       <c r="AB28" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC28" t="str">
-        <f t="shared" si="8"/>
-        <v>01000010</v>
+        <f>_xlfn.CONCAT(O18:O25)</f>
+        <v>00000010</v>
       </c>
       <c r="AD28" t="str">
-        <f t="shared" si="4"/>
-        <v>42</v>
+        <f t="shared" si="5"/>
+        <v>02</v>
       </c>
     </row>
     <row r="29" spans="2:34" x14ac:dyDescent="0.25">
@@ -5057,170 +5030,170 @@
         <v>30</v>
       </c>
       <c r="AB29" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC29" t="str">
-        <f t="shared" si="8"/>
-        <v>01000010</v>
+        <f>_xlfn.CONCAT(N18:N25)</f>
+        <v>00000010</v>
       </c>
       <c r="AD29" t="str">
-        <f t="shared" si="4"/>
-        <v>42</v>
+        <f t="shared" si="5"/>
+        <v>02</v>
       </c>
     </row>
     <row r="30" spans="2:34" x14ac:dyDescent="0.25">
       <c r="AB30" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC30" t="str">
-        <f t="shared" si="8"/>
-        <v>01000010</v>
+        <f>_xlfn.CONCAT(M18:M25)</f>
+        <v>00000010</v>
       </c>
       <c r="AD30" t="str">
-        <f t="shared" si="4"/>
-        <v>42</v>
+        <f t="shared" si="5"/>
+        <v>02</v>
       </c>
     </row>
     <row r="31" spans="2:34" x14ac:dyDescent="0.25">
       <c r="AB31" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC31" t="str">
-        <f t="shared" si="8"/>
-        <v>01000010</v>
+        <f>_xlfn.CONCAT(L18:L25)</f>
+        <v>00000010</v>
       </c>
       <c r="AD31" t="str">
-        <f t="shared" si="4"/>
-        <v>42</v>
+        <f t="shared" si="5"/>
+        <v>02</v>
       </c>
     </row>
     <row r="32" spans="2:34" x14ac:dyDescent="0.25">
       <c r="AB32" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC32" t="str">
-        <f t="shared" si="8"/>
-        <v>01111110</v>
+        <f>_xlfn.CONCAT(K18:K25)</f>
+        <v>11111110</v>
       </c>
       <c r="AD32" t="str">
-        <f t="shared" si="4"/>
-        <v>7E</v>
+        <f t="shared" si="5"/>
+        <v>FE</v>
       </c>
     </row>
     <row r="33" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB33" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC33" t="str">
-        <f t="shared" si="8"/>
+        <f>_xlfn.CONCAT(J18:J25)</f>
         <v>00000000</v>
       </c>
       <c r="AD33" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>00</v>
       </c>
     </row>
     <row r="34" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB34" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC34" t="str">
-        <f>_xlfn.CONCAT(J10:Q10)</f>
+        <f>_xlfn.CONCAT(Q10:Q17)</f>
         <v>01000010</v>
       </c>
       <c r="AD34" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>42</v>
       </c>
     </row>
     <row r="35" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB35" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC35" t="str">
-        <f t="shared" ref="AC35:AC41" si="9">_xlfn.CONCAT(J11:Q11)</f>
+        <f>_xlfn.CONCAT(P10:P17)</f>
         <v>11000011</v>
       </c>
       <c r="AD35" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>C3</v>
       </c>
     </row>
     <row r="36" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB36" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC36" t="str">
-        <f t="shared" si="9"/>
+        <f>_xlfn.CONCAT(O10:O17)</f>
         <v>00000000</v>
       </c>
       <c r="AD36" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>00</v>
       </c>
     </row>
     <row r="37" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB37" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC37" t="str">
-        <f t="shared" si="9"/>
+        <f>_xlfn.CONCAT(N10:N17)</f>
         <v>00000000</v>
       </c>
       <c r="AD37" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>00</v>
       </c>
     </row>
     <row r="38" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB38" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC38" t="str">
-        <f t="shared" si="9"/>
+        <f>_xlfn.CONCAT(M9:M16)</f>
         <v>00000000</v>
       </c>
       <c r="AD38" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>00</v>
       </c>
     </row>
     <row r="39" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB39" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC39" t="str">
-        <f t="shared" si="9"/>
+        <f>_xlfn.CONCAT(L10:L17)</f>
         <v>00000000</v>
       </c>
       <c r="AD39" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>00</v>
       </c>
     </row>
     <row r="40" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB40" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC40" t="str">
-        <f t="shared" si="9"/>
+        <f>_xlfn.CONCAT(K10:K17)</f>
         <v>11000011</v>
       </c>
       <c r="AD40" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>C3</v>
       </c>
     </row>
     <row r="41" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB41" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC41" t="str">
-        <f t="shared" si="9"/>
+        <f>_xlfn.CONCAT(J10:J17)</f>
         <v>01000010</v>
       </c>
       <c r="AD41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>42</v>
       </c>
     </row>
@@ -5263,10 +5236,10 @@
   <sheetData>
     <row r="1" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="AC1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="AD1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5310,18 +5283,15 @@
       <c r="W2" s="15"/>
       <c r="X2" s="15"/>
       <c r="Y2" s="17"/>
-      <c r="AA2" t="s">
-        <v>36</v>
-      </c>
       <c r="AB2" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC2" t="str">
-        <f>_xlfn.CONCAT(J2:Q2)</f>
+        <f>_xlfn.CONCAT(Q2:Q9)</f>
         <v>00000000</v>
       </c>
       <c r="AD2" t="str">
-        <f t="shared" ref="AD2:AD10" si="0">IF(BIN2DEC(AC2)&lt;16,"0","")&amp;BIN2HEX(AC2)</f>
+        <f t="shared" ref="AD2:AD9" si="0">IF(BIN2DEC(AC2)&lt;16,"0","")&amp;BIN2HEX(AC2)</f>
         <v>00</v>
       </c>
       <c r="AF2" t="s">
@@ -5333,7 +5303,7 @@
       </c>
       <c r="AH2" s="11" t="str">
         <f>_xlfn.TEXTJOIN(", ",TRUE,AG2:AG9)</f>
-        <v>0x0000, 0x0000, 0x3C3F, 0x2420, 0x2420, 0x243F, 0x2400, 0x2400</v>
+        <v>0x0000, 0x0000, 0x3F3C, 0x2024, 0x2024, 0x3F24, 0x0024, 0x0024</v>
       </c>
     </row>
     <row r="3" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5377,14 +5347,11 @@
       <c r="W3" s="19"/>
       <c r="X3" s="19"/>
       <c r="Y3" s="21"/>
-      <c r="AA3" t="s">
-        <v>33</v>
-      </c>
       <c r="AB3" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC3" t="str">
-        <f t="shared" ref="AC3:AC9" si="1">_xlfn.CONCAT(J3:Q3)</f>
+        <f>_xlfn.CONCAT(P2:P9)</f>
         <v>00000000</v>
       </c>
       <c r="AD3" t="str">
@@ -5392,7 +5359,7 @@
         <v>00</v>
       </c>
       <c r="AG3" t="str">
-        <f t="shared" ref="AG3:AG9" si="2">"0x"&amp;AD3&amp;AD11</f>
+        <f t="shared" ref="AG3:AG9" si="1">"0x"&amp;AD3&amp;AD11</f>
         <v>0x0000</v>
       </c>
     </row>
@@ -5438,19 +5405,19 @@
       <c r="X4" s="19"/>
       <c r="Y4" s="21"/>
       <c r="AB4" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC4" t="str">
-        <f t="shared" si="1"/>
-        <v>00111100</v>
+        <f>_xlfn.CONCAT(O2:O9)</f>
+        <v>00111111</v>
       </c>
       <c r="AD4" t="str">
         <f t="shared" si="0"/>
-        <v>3C</v>
+        <v>3F</v>
       </c>
       <c r="AG4" t="str">
-        <f t="shared" si="2"/>
-        <v>0x3C3F</v>
+        <f t="shared" si="1"/>
+        <v>0x3F3C</v>
       </c>
     </row>
     <row r="5" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5494,23 +5461,20 @@
       <c r="W5" s="19"/>
       <c r="X5" s="19"/>
       <c r="Y5" s="21"/>
-      <c r="AA5" t="s">
-        <v>34</v>
-      </c>
       <c r="AB5" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC5" t="str">
-        <f t="shared" si="1"/>
-        <v>00100100</v>
+        <f>_xlfn.CONCAT(N2:N9)</f>
+        <v>00100000</v>
       </c>
       <c r="AD5" t="str">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="AG5" t="str">
-        <f t="shared" si="2"/>
-        <v>0x2420</v>
+        <f t="shared" si="1"/>
+        <v>0x2024</v>
       </c>
     </row>
     <row r="6" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5555,19 +5519,19 @@
       <c r="X6" s="19"/>
       <c r="Y6" s="21"/>
       <c r="AB6" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC6" t="str">
-        <f t="shared" si="1"/>
-        <v>00100100</v>
+        <f>_xlfn.CONCAT(M2:M9)</f>
+        <v>00100000</v>
       </c>
       <c r="AD6" t="str">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="AG6" t="str">
-        <f t="shared" si="2"/>
-        <v>0x2420</v>
+        <f t="shared" si="1"/>
+        <v>0x2024</v>
       </c>
     </row>
     <row r="7" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5611,23 +5575,20 @@
       <c r="W7" s="19"/>
       <c r="X7" s="19"/>
       <c r="Y7" s="21"/>
-      <c r="AA7" t="s">
+      <c r="AB7" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="AB7" s="11" t="s">
-        <v>39</v>
-      </c>
       <c r="AC7" t="str">
-        <f t="shared" si="1"/>
-        <v>00100100</v>
+        <f>_xlfn.CONCAT(L2:L9)</f>
+        <v>00111111</v>
       </c>
       <c r="AD7" t="str">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>3F</v>
       </c>
       <c r="AG7" t="str">
-        <f t="shared" si="2"/>
-        <v>0x243F</v>
+        <f t="shared" si="1"/>
+        <v>0x3F24</v>
       </c>
     </row>
     <row r="8" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5672,19 +5633,19 @@
       <c r="X8" s="19"/>
       <c r="Y8" s="21"/>
       <c r="AB8" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC8" t="str">
-        <f t="shared" si="1"/>
-        <v>00100100</v>
+        <f>_xlfn.CONCAT(K2:K9)</f>
+        <v>00000000</v>
       </c>
       <c r="AD8" t="str">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>00</v>
       </c>
       <c r="AG8" t="str">
-        <f t="shared" si="2"/>
-        <v>0x2400</v>
+        <f t="shared" si="1"/>
+        <v>0x0024</v>
       </c>
     </row>
     <row r="9" spans="2:34" x14ac:dyDescent="0.25">
@@ -5729,19 +5690,19 @@
       <c r="X9" s="19"/>
       <c r="Y9" s="21"/>
       <c r="AB9" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC9" t="str">
-        <f t="shared" si="1"/>
-        <v>00100100</v>
+        <f>_xlfn.CONCAT(J2:J9)</f>
+        <v>00000000</v>
       </c>
       <c r="AD9" t="str">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>00</v>
       </c>
       <c r="AG9" t="str">
-        <f t="shared" si="2"/>
-        <v>0x2400</v>
+        <f t="shared" si="1"/>
+        <v>0x0024</v>
       </c>
     </row>
     <row r="10" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5818,26 +5779,26 @@
         <v>0</v>
       </c>
       <c r="AB10" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC10" t="str">
-        <f>_xlfn.CONCAT(B10:I10)</f>
+        <f>_xlfn.CONCAT(Y10:Y17)</f>
         <v>00000000</v>
       </c>
       <c r="AD10" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(BIN2DEC(AC10)&lt;16,"0","")&amp;BIN2HEX(AC10)</f>
         <v>00</v>
       </c>
       <c r="AF10" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="AG10" t="str">
         <f>"0x"&amp;AD18&amp;AD26</f>
-        <v>0x0024</v>
+        <v>0x2400</v>
       </c>
       <c r="AH10" s="12" t="str">
         <f>_xlfn.TEXTJOIN(", ",TRUE,AG10:AG17)</f>
-        <v>0x0024, 0x0024, 0xFC24, 0x0424, 0x0424, 0xFC3C, 0x0000, 0x0000</v>
+        <v>0x2400, 0x2400, 0x24FC, 0x2404, 0x2404, 0x3CFC, 0x0000, 0x0000</v>
       </c>
     </row>
     <row r="11" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5914,10 +5875,10 @@
         <v>0</v>
       </c>
       <c r="AB11" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC11" t="str">
-        <f t="shared" ref="AC11:AC17" si="3">_xlfn.CONCAT(B11:I11)</f>
+        <f>_xlfn.CONCAT(X10:X17)</f>
         <v>00000000</v>
       </c>
       <c r="AD11" t="str">
@@ -5926,7 +5887,7 @@
       </c>
       <c r="AG11" t="str">
         <f>"0x"&amp;AD19&amp;AD27</f>
-        <v>0x0024</v>
+        <v>0x2400</v>
       </c>
     </row>
     <row r="12" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6003,19 +5964,19 @@
         <v>0</v>
       </c>
       <c r="AB12" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC12" t="str">
-        <f t="shared" si="3"/>
-        <v>00111111</v>
+        <f>_xlfn.CONCAT(W10:W17)</f>
+        <v>00111100</v>
       </c>
       <c r="AD12" t="str">
-        <f t="shared" ref="AD12:AD41" si="4">IF(BIN2DEC(AC12)&lt;16,"0","")&amp;BIN2HEX(AC12)</f>
-        <v>3F</v>
+        <f>IF(BIN2DEC(AC12)&lt;16,"0","")&amp;BIN2HEX(AC12)</f>
+        <v>3C</v>
       </c>
       <c r="AG12" t="str">
         <f>"0x"&amp;AD20&amp;AD28</f>
-        <v>0xFC24</v>
+        <v>0x24FC</v>
       </c>
     </row>
     <row r="13" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6092,19 +6053,19 @@
         <v>0</v>
       </c>
       <c r="AB13" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC13" t="str">
-        <f t="shared" si="3"/>
-        <v>00100000</v>
+        <f>_xlfn.CONCAT(V10:V17)</f>
+        <v>00100100</v>
       </c>
       <c r="AD13" t="str">
-        <f t="shared" si="4"/>
-        <v>20</v>
+        <f>IF(BIN2DEC(AC13)&lt;16,"0","")&amp;BIN2HEX(AC13)</f>
+        <v>24</v>
       </c>
       <c r="AG13" t="str">
         <f>"0x"&amp;AD21&amp;AD29</f>
-        <v>0x0424</v>
+        <v>0x2404</v>
       </c>
     </row>
     <row r="14" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6181,19 +6142,19 @@
         <v>0</v>
       </c>
       <c r="AB14" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC14" t="str">
-        <f t="shared" si="3"/>
-        <v>00100000</v>
+        <f>_xlfn.CONCAT(U10:U17)</f>
+        <v>00100100</v>
       </c>
       <c r="AD14" t="str">
-        <f t="shared" si="4"/>
-        <v>20</v>
+        <f>IF(BIN2DEC(AC14)&lt;16,"0","")&amp;BIN2HEX(AC14)</f>
+        <v>24</v>
       </c>
       <c r="AG14" t="str">
         <f>"0x"&amp;AD22&amp;AD30</f>
-        <v>0x0424</v>
+        <v>0x2404</v>
       </c>
     </row>
     <row r="15" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6270,19 +6231,19 @@
         <v>0</v>
       </c>
       <c r="AB15" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC15" t="str">
-        <f t="shared" si="3"/>
-        <v>00111111</v>
+        <f>_xlfn.CONCAT(T10:T17)</f>
+        <v>00100100</v>
       </c>
       <c r="AD15" t="str">
-        <f t="shared" si="4"/>
-        <v>3F</v>
+        <f>IF(BIN2DEC(AC15)&lt;16,"0","")&amp;BIN2HEX(AC15)</f>
+        <v>24</v>
       </c>
       <c r="AG15" t="str">
         <f>"0x"&amp;AD23&amp;AD31</f>
-        <v>0xFC3C</v>
+        <v>0x3CFC</v>
       </c>
     </row>
     <row r="16" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6359,15 +6320,15 @@
         <v>0</v>
       </c>
       <c r="AB16" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC16" t="str">
-        <f t="shared" si="3"/>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(S10:S17)</f>
+        <v>00100100</v>
       </c>
       <c r="AD16" t="str">
-        <f t="shared" si="4"/>
-        <v>00</v>
+        <f>IF(BIN2DEC(AC16)&lt;16,"0","")&amp;BIN2HEX(AC16)</f>
+        <v>24</v>
       </c>
       <c r="AG16" t="str">
         <f>"0x"&amp;AD24&amp;AD32</f>
@@ -6448,15 +6409,15 @@
         <v>0</v>
       </c>
       <c r="AB17" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC17" t="str">
-        <f t="shared" si="3"/>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(R10:R17)</f>
+        <v>00100100</v>
       </c>
       <c r="AD17" t="str">
-        <f t="shared" si="4"/>
-        <v>00</v>
+        <f>IF(BIN2DEC(AC17)&lt;16,"0","")&amp;BIN2HEX(AC17)</f>
+        <v>24</v>
       </c>
       <c r="AG17" t="str">
         <f>"0x"&amp;AD25&amp;AD33</f>
@@ -6505,25 +6466,25 @@
       <c r="X18" s="19"/>
       <c r="Y18" s="21"/>
       <c r="AB18" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC18" t="str">
-        <f>_xlfn.CONCAT(R10:Y10)</f>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(I10:I17)</f>
+        <v>00100100</v>
       </c>
       <c r="AD18" t="str">
-        <f t="shared" si="4"/>
-        <v>00</v>
+        <f>IF(BIN2DEC(AC18)&lt;16,"0","")&amp;BIN2HEX(AC18)</f>
+        <v>24</v>
       </c>
       <c r="AF18" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="AG18" t="str">
         <f>"0x"&amp;AD34&amp;"00"</f>
         <v>0x2400</v>
       </c>
       <c r="AH18" s="10" t="str">
-        <f t="shared" ref="AH18" si="5">_xlfn.TEXTJOIN(", ",TRUE,AG18:AG25)</f>
+        <f t="shared" ref="AH18" si="2">_xlfn.TEXTJOIN(", ",TRUE,AG18:AG25)</f>
         <v>0x2400, 0x2400, 0xE700, 0x0000, 0x0000, 0xE700, 0x2400, 0x2400</v>
       </c>
     </row>
@@ -6569,18 +6530,18 @@
       <c r="X19" s="19"/>
       <c r="Y19" s="21"/>
       <c r="AB19" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC19" t="str">
-        <f t="shared" ref="AC19:AC25" si="6">_xlfn.CONCAT(R11:Y11)</f>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(H10:H17)</f>
+        <v>00100100</v>
       </c>
       <c r="AD19" t="str">
-        <f t="shared" si="4"/>
-        <v>00</v>
+        <f>IF(BIN2DEC(AC19)&lt;16,"0","")&amp;BIN2HEX(AC19)</f>
+        <v>24</v>
       </c>
       <c r="AG19" t="str">
-        <f t="shared" ref="AG19:AG25" si="7">"0x"&amp;AD35&amp;"00"</f>
+        <f t="shared" ref="AG19:AG25" si="3">"0x"&amp;AD35&amp;"00"</f>
         <v>0x2400</v>
       </c>
     </row>
@@ -6626,18 +6587,18 @@
       <c r="X20" s="19"/>
       <c r="Y20" s="21"/>
       <c r="AB20" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC20" t="str">
-        <f t="shared" si="6"/>
-        <v>11111100</v>
+        <f>_xlfn.CONCAT(G10:G17)</f>
+        <v>00100100</v>
       </c>
       <c r="AD20" t="str">
-        <f t="shared" si="4"/>
-        <v>FC</v>
+        <f>IF(BIN2DEC(AC20)&lt;16,"0","")&amp;BIN2HEX(AC20)</f>
+        <v>24</v>
       </c>
       <c r="AG20" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>0xE700</v>
       </c>
     </row>
@@ -6683,18 +6644,18 @@
       <c r="X21" s="19"/>
       <c r="Y21" s="21"/>
       <c r="AB21" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC21" t="str">
-        <f t="shared" si="6"/>
-        <v>00000100</v>
+        <f>_xlfn.CONCAT(F10:F17)</f>
+        <v>00100100</v>
       </c>
       <c r="AD21" t="str">
-        <f t="shared" si="4"/>
-        <v>04</v>
+        <f>IF(BIN2DEC(AC21)&lt;16,"0","")&amp;BIN2HEX(AC21)</f>
+        <v>24</v>
       </c>
       <c r="AG21" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>0x0000</v>
       </c>
     </row>
@@ -6740,18 +6701,18 @@
       <c r="X22" s="19"/>
       <c r="Y22" s="21"/>
       <c r="AB22" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC22" t="str">
-        <f t="shared" si="6"/>
-        <v>00000100</v>
+        <f>_xlfn.CONCAT(E10:E17)</f>
+        <v>00100100</v>
       </c>
       <c r="AD22" t="str">
-        <f t="shared" si="4"/>
-        <v>04</v>
+        <f>IF(BIN2DEC(AC22)&lt;16,"0","")&amp;BIN2HEX(AC22)</f>
+        <v>24</v>
       </c>
       <c r="AG22" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>0x0000</v>
       </c>
     </row>
@@ -6797,18 +6758,18 @@
       <c r="X23" s="19"/>
       <c r="Y23" s="21"/>
       <c r="AB23" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC23" t="str">
-        <f t="shared" si="6"/>
-        <v>11111100</v>
+        <f>_xlfn.CONCAT(D10:D17)</f>
+        <v>00111100</v>
       </c>
       <c r="AD23" t="str">
-        <f t="shared" si="4"/>
-        <v>FC</v>
+        <f>IF(BIN2DEC(AC23)&lt;16,"0","")&amp;BIN2HEX(AC23)</f>
+        <v>3C</v>
       </c>
       <c r="AG23" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>0xE700</v>
       </c>
     </row>
@@ -6854,18 +6815,18 @@
       <c r="X24" s="19"/>
       <c r="Y24" s="21"/>
       <c r="AB24" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC24" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.CONCAT(C10:C17)</f>
         <v>00000000</v>
       </c>
       <c r="AD24" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(BIN2DEC(AC24)&lt;16,"0","")&amp;BIN2HEX(AC24)</f>
         <v>00</v>
       </c>
       <c r="AG24" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>0x2400</v>
       </c>
     </row>
@@ -6911,32 +6872,32 @@
       <c r="X25" s="25"/>
       <c r="Y25" s="27"/>
       <c r="AB25" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC25" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.CONCAT(B10:B17)</f>
         <v>00000000</v>
       </c>
       <c r="AD25" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(BIN2DEC(AC25)&lt;16,"0","")&amp;BIN2HEX(AC25)</f>
         <v>00</v>
       </c>
       <c r="AG25" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>0x2400</v>
       </c>
     </row>
     <row r="26" spans="2:34" x14ac:dyDescent="0.25">
       <c r="AB26" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC26" t="str">
-        <f>_xlfn.CONCAT(J18:Q18)</f>
-        <v>00100100</v>
+        <f>_xlfn.CONCAT(Q18:Q25)</f>
+        <v>00000000</v>
       </c>
       <c r="AD26" t="str">
-        <f t="shared" si="4"/>
-        <v>24</v>
+        <f t="shared" ref="AD26:AD41" si="4">IF(BIN2DEC(AC26)&lt;16,"0","")&amp;BIN2HEX(AC26)</f>
+        <v>00</v>
       </c>
       <c r="AH26" s="13"/>
     </row>
@@ -6945,37 +6906,40 @@
         <v>28</v>
       </c>
       <c r="AB27" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC27" t="str">
-        <f t="shared" ref="AC27:AC33" si="8">_xlfn.CONCAT(J19:Q19)</f>
-        <v>00100100</v>
+        <f>_xlfn.CONCAT(P18:P25)</f>
+        <v>00000000</v>
       </c>
       <c r="AD27" t="str">
         <f t="shared" si="4"/>
-        <v>24</v>
+        <v>00</v>
       </c>
     </row>
     <row r="28" spans="2:34" x14ac:dyDescent="0.25">
-      <c r="L28" s="11" t="s">
+      <c r="L28" s="12" t="s">
         <v>31</v>
       </c>
       <c r="M28" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="O28" s="9" t="s">
+      <c r="O28" s="11" t="s">
         <v>32</v>
       </c>
+      <c r="Q28" t="s">
+        <v>43</v>
+      </c>
       <c r="AB28" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC28" t="str">
-        <f t="shared" si="8"/>
-        <v>00100100</v>
+        <f>_xlfn.CONCAT(O18:O25)</f>
+        <v>11111100</v>
       </c>
       <c r="AD28" t="str">
         <f t="shared" si="4"/>
-        <v>24</v>
+        <v>FC</v>
       </c>
     </row>
     <row r="29" spans="2:34" x14ac:dyDescent="0.25">
@@ -6983,49 +6947,49 @@
         <v>30</v>
       </c>
       <c r="AB29" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC29" t="str">
-        <f t="shared" si="8"/>
-        <v>00100100</v>
+        <f>_xlfn.CONCAT(N18:N25)</f>
+        <v>00000100</v>
       </c>
       <c r="AD29" t="str">
         <f t="shared" si="4"/>
-        <v>24</v>
+        <v>04</v>
       </c>
     </row>
     <row r="30" spans="2:34" x14ac:dyDescent="0.25">
       <c r="AB30" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC30" t="str">
-        <f t="shared" si="8"/>
-        <v>00100100</v>
+        <f>_xlfn.CONCAT(M18:M25)</f>
+        <v>00000100</v>
       </c>
       <c r="AD30" t="str">
         <f t="shared" si="4"/>
-        <v>24</v>
+        <v>04</v>
       </c>
     </row>
     <row r="31" spans="2:34" x14ac:dyDescent="0.25">
       <c r="AB31" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC31" t="str">
-        <f t="shared" si="8"/>
-        <v>00111100</v>
+        <f>_xlfn.CONCAT(L18:L25)</f>
+        <v>11111100</v>
       </c>
       <c r="AD31" t="str">
         <f t="shared" si="4"/>
-        <v>3C</v>
+        <v>FC</v>
       </c>
     </row>
     <row r="32" spans="2:34" x14ac:dyDescent="0.25">
       <c r="AB32" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC32" t="str">
-        <f t="shared" si="8"/>
+        <f>_xlfn.CONCAT(K18:K25)</f>
         <v>00000000</v>
       </c>
       <c r="AD32" t="str">
@@ -7035,10 +6999,10 @@
     </row>
     <row r="33" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB33" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC33" t="str">
-        <f t="shared" si="8"/>
+        <f>_xlfn.CONCAT(J18:J25)</f>
         <v>00000000</v>
       </c>
       <c r="AD33" t="str">
@@ -7048,10 +7012,10 @@
     </row>
     <row r="34" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB34" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC34" t="str">
-        <f>_xlfn.CONCAT(J10:Q10)</f>
+        <f>_xlfn.CONCAT(Q10:Q17)</f>
         <v>00100100</v>
       </c>
       <c r="AD34" t="str">
@@ -7061,10 +7025,10 @@
     </row>
     <row r="35" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB35" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC35" t="str">
-        <f t="shared" ref="AC35:AC41" si="9">_xlfn.CONCAT(J11:Q11)</f>
+        <f>_xlfn.CONCAT(P10:P17)</f>
         <v>00100100</v>
       </c>
       <c r="AD35" t="str">
@@ -7074,10 +7038,10 @@
     </row>
     <row r="36" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB36" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC36" t="str">
-        <f t="shared" si="9"/>
+        <f>_xlfn.CONCAT(O10:O17)</f>
         <v>11100111</v>
       </c>
       <c r="AD36" t="str">
@@ -7087,10 +7051,10 @@
     </row>
     <row r="37" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB37" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC37" t="str">
-        <f t="shared" si="9"/>
+        <f>_xlfn.CONCAT(N10:N17)</f>
         <v>00000000</v>
       </c>
       <c r="AD37" t="str">
@@ -7100,10 +7064,10 @@
     </row>
     <row r="38" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB38" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC38" t="str">
-        <f t="shared" si="9"/>
+        <f>_xlfn.CONCAT(M9:M16)</f>
         <v>00000000</v>
       </c>
       <c r="AD38" t="str">
@@ -7113,10 +7077,10 @@
     </row>
     <row r="39" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB39" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC39" t="str">
-        <f t="shared" si="9"/>
+        <f>_xlfn.CONCAT(L10:L17)</f>
         <v>11100111</v>
       </c>
       <c r="AD39" t="str">
@@ -7126,10 +7090,10 @@
     </row>
     <row r="40" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB40" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC40" t="str">
-        <f t="shared" si="9"/>
+        <f>_xlfn.CONCAT(K10:K17)</f>
         <v>00100100</v>
       </c>
       <c r="AD40" t="str">
@@ -7139,10 +7103,10 @@
     </row>
     <row r="41" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB41" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC41" t="str">
-        <f t="shared" si="9"/>
+        <f>_xlfn.CONCAT(J10:J17)</f>
         <v>00100100</v>
       </c>
       <c r="AD41" t="str">
@@ -7161,10 +7125,10 @@
     <mergeCell ref="R18:Y25"/>
   </mergeCells>
   <conditionalFormatting sqref="B2:Y25">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="0">
+    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="0">
       <formula>NOT(ISERROR(SEARCH("0",B2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7189,10 +7153,10 @@
   <sheetData>
     <row r="1" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="AC1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="AD1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -7236,18 +7200,15 @@
       <c r="W2" s="15"/>
       <c r="X2" s="15"/>
       <c r="Y2" s="17"/>
-      <c r="AA2" t="s">
-        <v>36</v>
-      </c>
       <c r="AB2" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC2" t="str">
-        <f>_xlfn.CONCAT(J2:Q2)</f>
+        <f>_xlfn.CONCAT(Q2:Q9)</f>
         <v>00000000</v>
       </c>
       <c r="AD2" t="str">
-        <f t="shared" ref="AD2:AD10" si="0">IF(BIN2DEC(AC2)&lt;16,"0","")&amp;BIN2HEX(AC2)</f>
+        <f t="shared" ref="AD2:AD9" si="0">IF(BIN2DEC(AC2)&lt;16,"0","")&amp;BIN2HEX(AC2)</f>
         <v>00</v>
       </c>
       <c r="AF2" t="s">
@@ -7259,7 +7220,7 @@
       </c>
       <c r="AH2" s="11" t="str">
         <f>_xlfn.TEXTJOIN(", ",TRUE,AG2:AG9)</f>
-        <v>0x0000, 0x0000, 0x0000, 0x0000, 0x0000, 0x0000, 0x0000, 0x0000</v>
+        <v>0x0000, 0x0000, 0x0000, 0x1F18, 0x1F18, 0x0018, 0x0018, 0x0018</v>
       </c>
     </row>
     <row r="3" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -7303,14 +7264,11 @@
       <c r="W3" s="19"/>
       <c r="X3" s="19"/>
       <c r="Y3" s="21"/>
-      <c r="AA3" t="s">
-        <v>33</v>
-      </c>
       <c r="AB3" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC3" t="str">
-        <f t="shared" ref="AC3:AC9" si="1">_xlfn.CONCAT(J3:Q3)</f>
+        <f>_xlfn.CONCAT(P2:P9)</f>
         <v>00000000</v>
       </c>
       <c r="AD3" t="str">
@@ -7318,7 +7276,7 @@
         <v>00</v>
       </c>
       <c r="AG3" t="str">
-        <f t="shared" ref="AG3:AG9" si="2">"0x"&amp;AD3&amp;AD11</f>
+        <f t="shared" ref="AG3:AG9" si="1">"0x"&amp;AD3&amp;AD11</f>
         <v>0x0000</v>
       </c>
     </row>
@@ -7364,10 +7322,10 @@
       <c r="X4" s="19"/>
       <c r="Y4" s="21"/>
       <c r="AB4" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC4" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.CONCAT(O2:O9)</f>
         <v>00000000</v>
       </c>
       <c r="AD4" t="str">
@@ -7375,7 +7333,7 @@
         <v>00</v>
       </c>
       <c r="AG4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0x0000</v>
       </c>
     </row>
@@ -7398,10 +7356,10 @@
         <v>0</v>
       </c>
       <c r="M5" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N5" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O5" s="20">
         <v>0</v>
@@ -7420,23 +7378,20 @@
       <c r="W5" s="19"/>
       <c r="X5" s="19"/>
       <c r="Y5" s="21"/>
-      <c r="AA5" t="s">
-        <v>34</v>
-      </c>
       <c r="AB5" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC5" t="str">
-        <f t="shared" si="1"/>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(N2:N9)</f>
+        <v>00011111</v>
       </c>
       <c r="AD5" t="str">
         <f t="shared" si="0"/>
-        <v>00</v>
+        <v>1F</v>
       </c>
       <c r="AG5" t="str">
-        <f t="shared" si="2"/>
-        <v>0x0000</v>
+        <f t="shared" si="1"/>
+        <v>0x1F18</v>
       </c>
     </row>
     <row r="6" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -7458,10 +7413,10 @@
         <v>0</v>
       </c>
       <c r="M6" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N6" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O6" s="20">
         <v>0</v>
@@ -7481,19 +7436,19 @@
       <c r="X6" s="19"/>
       <c r="Y6" s="21"/>
       <c r="AB6" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC6" t="str">
-        <f t="shared" si="1"/>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(M2:M9)</f>
+        <v>00011111</v>
       </c>
       <c r="AD6" t="str">
         <f t="shared" si="0"/>
-        <v>00</v>
+        <v>1F</v>
       </c>
       <c r="AG6" t="str">
-        <f t="shared" si="2"/>
-        <v>0x0000</v>
+        <f t="shared" si="1"/>
+        <v>0x1F18</v>
       </c>
     </row>
     <row r="7" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -7515,10 +7470,10 @@
         <v>0</v>
       </c>
       <c r="M7" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N7" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O7" s="20">
         <v>0</v>
@@ -7537,14 +7492,11 @@
       <c r="W7" s="19"/>
       <c r="X7" s="19"/>
       <c r="Y7" s="21"/>
-      <c r="AA7" t="s">
+      <c r="AB7" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="AB7" s="11" t="s">
-        <v>39</v>
-      </c>
       <c r="AC7" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.CONCAT(L2:L9)</f>
         <v>00000000</v>
       </c>
       <c r="AD7" t="str">
@@ -7552,8 +7504,8 @@
         <v>00</v>
       </c>
       <c r="AG7" t="str">
-        <f t="shared" si="2"/>
-        <v>0x0000</v>
+        <f t="shared" si="1"/>
+        <v>0x0018</v>
       </c>
     </row>
     <row r="8" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -7575,10 +7527,10 @@
         <v>0</v>
       </c>
       <c r="M8" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N8" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O8" s="20">
         <v>0</v>
@@ -7598,10 +7550,10 @@
       <c r="X8" s="19"/>
       <c r="Y8" s="21"/>
       <c r="AB8" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC8" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.CONCAT(K2:K9)</f>
         <v>00000000</v>
       </c>
       <c r="AD8" t="str">
@@ -7609,8 +7561,8 @@
         <v>00</v>
       </c>
       <c r="AG8" t="str">
-        <f t="shared" si="2"/>
-        <v>0x0000</v>
+        <f t="shared" si="1"/>
+        <v>0x0018</v>
       </c>
     </row>
     <row r="9" spans="2:34" x14ac:dyDescent="0.25">
@@ -7632,10 +7584,10 @@
         <v>0</v>
       </c>
       <c r="M9" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N9" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O9" s="20">
         <v>0</v>
@@ -7655,10 +7607,10 @@
       <c r="X9" s="19"/>
       <c r="Y9" s="21"/>
       <c r="AB9" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC9" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.CONCAT(J2:J9)</f>
         <v>00000000</v>
       </c>
       <c r="AD9" t="str">
@@ -7666,8 +7618,8 @@
         <v>00</v>
       </c>
       <c r="AG9" t="str">
-        <f t="shared" si="2"/>
-        <v>0x0000</v>
+        <f t="shared" si="1"/>
+        <v>0x0018</v>
       </c>
     </row>
     <row r="10" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -7705,10 +7657,10 @@
         <v>0</v>
       </c>
       <c r="M10" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N10" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O10" s="20">
         <v>0</v>
@@ -7744,26 +7696,26 @@
         <v>0</v>
       </c>
       <c r="AB10" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC10" t="str">
-        <f>_xlfn.CONCAT(B10:I10)</f>
+        <f>_xlfn.CONCAT(Y10:Y17)</f>
         <v>00000000</v>
       </c>
       <c r="AD10" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(BIN2DEC(AC10)&lt;16,"0","")&amp;BIN2HEX(AC10)</f>
         <v>00</v>
       </c>
       <c r="AF10" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="AG10" t="str">
         <f>"0x"&amp;AD18&amp;AD26</f>
-        <v>0x0000</v>
+        <v>0x1800</v>
       </c>
       <c r="AH10" s="12" t="str">
         <f>_xlfn.TEXTJOIN(", ",TRUE,AG10:AG17)</f>
-        <v>0x0000, 0x0000, 0x0000, 0x0000, 0x0000, 0x0000, 0x0000, 0x0000</v>
+        <v>0x1800, 0x1800, 0x1800, 0x18F8, 0x18F8, 0x0000, 0x0000, 0x0000</v>
       </c>
     </row>
     <row r="11" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -7801,10 +7753,10 @@
         <v>0</v>
       </c>
       <c r="M11" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N11" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O11" s="20">
         <v>0</v>
@@ -7840,10 +7792,10 @@
         <v>0</v>
       </c>
       <c r="AB11" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC11" t="str">
-        <f t="shared" ref="AC11:AC17" si="3">_xlfn.CONCAT(B11:I11)</f>
+        <f>_xlfn.CONCAT(X10:X17)</f>
         <v>00000000</v>
       </c>
       <c r="AD11" t="str">
@@ -7852,7 +7804,7 @@
       </c>
       <c r="AG11" t="str">
         <f>"0x"&amp;AD19&amp;AD27</f>
-        <v>0x0000</v>
+        <v>0x1800</v>
       </c>
     </row>
     <row r="12" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -7890,10 +7842,10 @@
         <v>0</v>
       </c>
       <c r="M12" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N12" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O12" s="20">
         <v>0</v>
@@ -7929,19 +7881,19 @@
         <v>0</v>
       </c>
       <c r="AB12" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC12" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.CONCAT(W10:W17)</f>
         <v>00000000</v>
       </c>
       <c r="AD12" t="str">
-        <f t="shared" ref="AD12:AD41" si="4">IF(BIN2DEC(AC12)&lt;16,"0","")&amp;BIN2HEX(AC12)</f>
+        <f>IF(BIN2DEC(AC12)&lt;16,"0","")&amp;BIN2HEX(AC12)</f>
         <v>00</v>
       </c>
       <c r="AG12" t="str">
         <f>"0x"&amp;AD20&amp;AD28</f>
-        <v>0x0000</v>
+        <v>0x1800</v>
       </c>
     </row>
     <row r="13" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -7955,58 +7907,58 @@
         <v>0</v>
       </c>
       <c r="E13" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H13" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K13" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L13" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M13" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N13" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O13" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P13" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q13" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R13" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S13" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T13" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U13" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V13" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W13" s="20">
         <v>0</v>
@@ -8018,19 +7970,19 @@
         <v>0</v>
       </c>
       <c r="AB13" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC13" t="str">
-        <f t="shared" si="3"/>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(V10:V17)</f>
+        <v>00011000</v>
       </c>
       <c r="AD13" t="str">
-        <f t="shared" si="4"/>
-        <v>00</v>
+        <f>IF(BIN2DEC(AC13)&lt;16,"0","")&amp;BIN2HEX(AC13)</f>
+        <v>18</v>
       </c>
       <c r="AG13" t="str">
         <f>"0x"&amp;AD21&amp;AD29</f>
-        <v>0x0000</v>
+        <v>0x18F8</v>
       </c>
     </row>
     <row r="14" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -8044,58 +7996,58 @@
         <v>0</v>
       </c>
       <c r="E14" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K14" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L14" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M14" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N14" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O14" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P14" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q14" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R14" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S14" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T14" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U14" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V14" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W14" s="20">
         <v>0</v>
@@ -8107,19 +8059,19 @@
         <v>0</v>
       </c>
       <c r="AB14" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC14" t="str">
-        <f t="shared" si="3"/>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(U10:U17)</f>
+        <v>00011000</v>
       </c>
       <c r="AD14" t="str">
-        <f t="shared" si="4"/>
-        <v>00</v>
+        <f>IF(BIN2DEC(AC14)&lt;16,"0","")&amp;BIN2HEX(AC14)</f>
+        <v>18</v>
       </c>
       <c r="AG14" t="str">
         <f>"0x"&amp;AD22&amp;AD30</f>
-        <v>0x0000</v>
+        <v>0x18F8</v>
       </c>
     </row>
     <row r="15" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -8157,10 +8109,10 @@
         <v>0</v>
       </c>
       <c r="M15" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N15" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O15" s="20">
         <v>0</v>
@@ -8196,15 +8148,15 @@
         <v>0</v>
       </c>
       <c r="AB15" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC15" t="str">
-        <f t="shared" si="3"/>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(T10:T17)</f>
+        <v>00011000</v>
       </c>
       <c r="AD15" t="str">
-        <f t="shared" si="4"/>
-        <v>00</v>
+        <f>IF(BIN2DEC(AC15)&lt;16,"0","")&amp;BIN2HEX(AC15)</f>
+        <v>18</v>
       </c>
       <c r="AG15" t="str">
         <f>"0x"&amp;AD23&amp;AD31</f>
@@ -8246,10 +8198,10 @@
         <v>0</v>
       </c>
       <c r="M16" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N16" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O16" s="20">
         <v>0</v>
@@ -8285,15 +8237,15 @@
         <v>0</v>
       </c>
       <c r="AB16" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC16" t="str">
-        <f t="shared" si="3"/>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(S10:S17)</f>
+        <v>00011000</v>
       </c>
       <c r="AD16" t="str">
-        <f t="shared" si="4"/>
-        <v>00</v>
+        <f>IF(BIN2DEC(AC16)&lt;16,"0","")&amp;BIN2HEX(AC16)</f>
+        <v>18</v>
       </c>
       <c r="AG16" t="str">
         <f>"0x"&amp;AD24&amp;AD32</f>
@@ -8335,10 +8287,10 @@
         <v>0</v>
       </c>
       <c r="M17" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N17" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O17" s="20">
         <v>0</v>
@@ -8374,15 +8326,15 @@
         <v>0</v>
       </c>
       <c r="AB17" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AC17" t="str">
-        <f t="shared" si="3"/>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(R10:R17)</f>
+        <v>00011000</v>
       </c>
       <c r="AD17" t="str">
-        <f t="shared" si="4"/>
-        <v>00</v>
+        <f>IF(BIN2DEC(AC17)&lt;16,"0","")&amp;BIN2HEX(AC17)</f>
+        <v>18</v>
       </c>
       <c r="AG17" t="str">
         <f>"0x"&amp;AD25&amp;AD33</f>
@@ -8408,10 +8360,10 @@
         <v>0</v>
       </c>
       <c r="M18" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N18" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O18" s="20">
         <v>0</v>
@@ -8431,26 +8383,26 @@
       <c r="X18" s="19"/>
       <c r="Y18" s="21"/>
       <c r="AB18" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC18" t="str">
-        <f>_xlfn.CONCAT(R10:Y10)</f>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(I10:I17)</f>
+        <v>00011000</v>
       </c>
       <c r="AD18" t="str">
-        <f t="shared" si="4"/>
-        <v>00</v>
+        <f>IF(BIN2DEC(AC18)&lt;16,"0","")&amp;BIN2HEX(AC18)</f>
+        <v>18</v>
       </c>
       <c r="AF18" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="AG18" t="str">
         <f>"0x"&amp;AD34&amp;"00"</f>
-        <v>0x0000</v>
+        <v>0x1800</v>
       </c>
       <c r="AH18" s="10" t="str">
-        <f t="shared" ref="AH18" si="5">_xlfn.TEXTJOIN(", ",TRUE,AG18:AG25)</f>
-        <v>0x0000, 0x0000, 0x0000, 0x0000, 0x0000, 0x0000, 0x0000, 0x0000</v>
+        <f t="shared" ref="AH18" si="2">_xlfn.TEXTJOIN(", ",TRUE,AG18:AG25)</f>
+        <v>0x1800, 0x1800, 0x1800, 0xFF00, 0xFF00, 0x1800, 0x1800, 0x1800</v>
       </c>
     </row>
     <row r="19" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -8472,10 +8424,10 @@
         <v>0</v>
       </c>
       <c r="M19" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N19" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O19" s="20">
         <v>0</v>
@@ -8495,19 +8447,19 @@
       <c r="X19" s="19"/>
       <c r="Y19" s="21"/>
       <c r="AB19" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC19" t="str">
-        <f t="shared" ref="AC19:AC25" si="6">_xlfn.CONCAT(R11:Y11)</f>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(H10:H17)</f>
+        <v>00011000</v>
       </c>
       <c r="AD19" t="str">
-        <f t="shared" si="4"/>
-        <v>00</v>
+        <f>IF(BIN2DEC(AC19)&lt;16,"0","")&amp;BIN2HEX(AC19)</f>
+        <v>18</v>
       </c>
       <c r="AG19" t="str">
-        <f t="shared" ref="AG19:AG25" si="7">"0x"&amp;AD35&amp;"00"</f>
-        <v>0x0000</v>
+        <f t="shared" ref="AG19:AG25" si="3">"0x"&amp;AD35&amp;"00"</f>
+        <v>0x1800</v>
       </c>
     </row>
     <row r="20" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -8529,10 +8481,10 @@
         <v>0</v>
       </c>
       <c r="M20" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N20" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O20" s="20">
         <v>0</v>
@@ -8552,19 +8504,19 @@
       <c r="X20" s="19"/>
       <c r="Y20" s="21"/>
       <c r="AB20" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC20" t="str">
-        <f t="shared" si="6"/>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(G10:G17)</f>
+        <v>00011000</v>
       </c>
       <c r="AD20" t="str">
-        <f t="shared" si="4"/>
-        <v>00</v>
+        <f>IF(BIN2DEC(AC20)&lt;16,"0","")&amp;BIN2HEX(AC20)</f>
+        <v>18</v>
       </c>
       <c r="AG20" t="str">
-        <f t="shared" si="7"/>
-        <v>0x0000</v>
+        <f t="shared" si="3"/>
+        <v>0x1800</v>
       </c>
     </row>
     <row r="21" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -8586,10 +8538,10 @@
         <v>0</v>
       </c>
       <c r="M21" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N21" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O21" s="20">
         <v>0</v>
@@ -8609,19 +8561,19 @@
       <c r="X21" s="19"/>
       <c r="Y21" s="21"/>
       <c r="AB21" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC21" t="str">
-        <f t="shared" si="6"/>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(F10:F17)</f>
+        <v>00011000</v>
       </c>
       <c r="AD21" t="str">
-        <f t="shared" si="4"/>
-        <v>00</v>
+        <f>IF(BIN2DEC(AC21)&lt;16,"0","")&amp;BIN2HEX(AC21)</f>
+        <v>18</v>
       </c>
       <c r="AG21" t="str">
-        <f t="shared" si="7"/>
-        <v>0x0000</v>
+        <f t="shared" si="3"/>
+        <v>0xFF00</v>
       </c>
     </row>
     <row r="22" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -8643,10 +8595,10 @@
         <v>0</v>
       </c>
       <c r="M22" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N22" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O22" s="20">
         <v>0</v>
@@ -8666,19 +8618,19 @@
       <c r="X22" s="19"/>
       <c r="Y22" s="21"/>
       <c r="AB22" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC22" t="str">
-        <f t="shared" si="6"/>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(E10:E17)</f>
+        <v>00011000</v>
       </c>
       <c r="AD22" t="str">
-        <f t="shared" si="4"/>
-        <v>00</v>
+        <f>IF(BIN2DEC(AC22)&lt;16,"0","")&amp;BIN2HEX(AC22)</f>
+        <v>18</v>
       </c>
       <c r="AG22" t="str">
-        <f t="shared" si="7"/>
-        <v>0x0000</v>
+        <f t="shared" si="3"/>
+        <v>0xFF00</v>
       </c>
     </row>
     <row r="23" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -8723,19 +8675,19 @@
       <c r="X23" s="19"/>
       <c r="Y23" s="21"/>
       <c r="AB23" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC23" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.CONCAT(D10:D17)</f>
         <v>00000000</v>
       </c>
       <c r="AD23" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(BIN2DEC(AC23)&lt;16,"0","")&amp;BIN2HEX(AC23)</f>
         <v>00</v>
       </c>
       <c r="AG23" t="str">
-        <f t="shared" si="7"/>
-        <v>0x0000</v>
+        <f t="shared" si="3"/>
+        <v>0x1800</v>
       </c>
     </row>
     <row r="24" spans="2:34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -8780,19 +8732,19 @@
       <c r="X24" s="19"/>
       <c r="Y24" s="21"/>
       <c r="AB24" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC24" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.CONCAT(C10:C17)</f>
         <v>00000000</v>
       </c>
       <c r="AD24" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(BIN2DEC(AC24)&lt;16,"0","")&amp;BIN2HEX(AC24)</f>
         <v>00</v>
       </c>
       <c r="AG24" t="str">
-        <f t="shared" si="7"/>
-        <v>0x0000</v>
+        <f t="shared" si="3"/>
+        <v>0x1800</v>
       </c>
     </row>
     <row r="25" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -8837,31 +8789,31 @@
       <c r="X25" s="25"/>
       <c r="Y25" s="27"/>
       <c r="AB25" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="AC25" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.CONCAT(B10:B17)</f>
         <v>00000000</v>
       </c>
       <c r="AD25" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(BIN2DEC(AC25)&lt;16,"0","")&amp;BIN2HEX(AC25)</f>
         <v>00</v>
       </c>
       <c r="AG25" t="str">
-        <f t="shared" si="7"/>
-        <v>0x0000</v>
+        <f t="shared" si="3"/>
+        <v>0x1800</v>
       </c>
     </row>
     <row r="26" spans="2:34" x14ac:dyDescent="0.25">
       <c r="AB26" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC26" t="str">
-        <f>_xlfn.CONCAT(J18:Q18)</f>
+        <f>_xlfn.CONCAT(Q18:Q25)</f>
         <v>00000000</v>
       </c>
       <c r="AD26" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="AD26:AD41" si="4">IF(BIN2DEC(AC26)&lt;16,"0","")&amp;BIN2HEX(AC26)</f>
         <v>00</v>
       </c>
       <c r="AH26" s="13"/>
@@ -8871,10 +8823,10 @@
         <v>28</v>
       </c>
       <c r="AB27" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC27" t="str">
-        <f t="shared" ref="AC27:AC33" si="8">_xlfn.CONCAT(J19:Q19)</f>
+        <f>_xlfn.CONCAT(P18:P25)</f>
         <v>00000000</v>
       </c>
       <c r="AD27" t="str">
@@ -8883,20 +8835,23 @@
       </c>
     </row>
     <row r="28" spans="2:34" x14ac:dyDescent="0.25">
-      <c r="L28" s="11" t="s">
+      <c r="L28" s="12" t="s">
         <v>31</v>
       </c>
       <c r="M28" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="O28" s="9" t="s">
+      <c r="O28" s="11" t="s">
         <v>32</v>
       </c>
+      <c r="Q28" t="s">
+        <v>43</v>
+      </c>
       <c r="AB28" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC28" t="str">
-        <f t="shared" si="8"/>
+        <f>_xlfn.CONCAT(O18:O25)</f>
         <v>00000000</v>
       </c>
       <c r="AD28" t="str">
@@ -8909,36 +8864,36 @@
         <v>30</v>
       </c>
       <c r="AB29" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC29" t="str">
-        <f t="shared" si="8"/>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(N18:N25)</f>
+        <v>11111000</v>
       </c>
       <c r="AD29" t="str">
         <f t="shared" si="4"/>
-        <v>00</v>
+        <v>F8</v>
       </c>
     </row>
     <row r="30" spans="2:34" x14ac:dyDescent="0.25">
       <c r="AB30" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC30" t="str">
-        <f t="shared" si="8"/>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(M18:M25)</f>
+        <v>11111000</v>
       </c>
       <c r="AD30" t="str">
         <f t="shared" si="4"/>
-        <v>00</v>
+        <v>F8</v>
       </c>
     </row>
     <row r="31" spans="2:34" x14ac:dyDescent="0.25">
       <c r="AB31" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC31" t="str">
-        <f t="shared" si="8"/>
+        <f>_xlfn.CONCAT(L18:L25)</f>
         <v>00000000</v>
       </c>
       <c r="AD31" t="str">
@@ -8948,10 +8903,10 @@
     </row>
     <row r="32" spans="2:34" x14ac:dyDescent="0.25">
       <c r="AB32" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC32" t="str">
-        <f t="shared" si="8"/>
+        <f>_xlfn.CONCAT(K18:K25)</f>
         <v>00000000</v>
       </c>
       <c r="AD32" t="str">
@@ -8961,10 +8916,10 @@
     </row>
     <row r="33" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB33" s="12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AC33" t="str">
-        <f t="shared" si="8"/>
+        <f>_xlfn.CONCAT(J18:J25)</f>
         <v>00000000</v>
       </c>
       <c r="AD33" t="str">
@@ -8974,106 +8929,106 @@
     </row>
     <row r="34" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB34" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC34" t="str">
-        <f>_xlfn.CONCAT(J10:Q10)</f>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(Q10:Q17)</f>
+        <v>00011000</v>
       </c>
       <c r="AD34" t="str">
         <f t="shared" si="4"/>
-        <v>00</v>
+        <v>18</v>
       </c>
     </row>
     <row r="35" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB35" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC35" t="str">
-        <f t="shared" ref="AC35:AC41" si="9">_xlfn.CONCAT(J11:Q11)</f>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(P10:P17)</f>
+        <v>00011000</v>
       </c>
       <c r="AD35" t="str">
         <f t="shared" si="4"/>
-        <v>00</v>
+        <v>18</v>
       </c>
     </row>
     <row r="36" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB36" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC36" t="str">
-        <f t="shared" si="9"/>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(O10:O17)</f>
+        <v>00011000</v>
       </c>
       <c r="AD36" t="str">
         <f t="shared" si="4"/>
-        <v>00</v>
+        <v>18</v>
       </c>
     </row>
     <row r="37" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB37" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC37" t="str">
-        <f t="shared" si="9"/>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(N10:N17)</f>
+        <v>11111111</v>
       </c>
       <c r="AD37" t="str">
         <f t="shared" si="4"/>
-        <v>00</v>
+        <v>FF</v>
       </c>
     </row>
     <row r="38" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB38" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC38" t="str">
-        <f t="shared" si="9"/>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(M9:M16)</f>
+        <v>11111111</v>
       </c>
       <c r="AD38" t="str">
         <f t="shared" si="4"/>
-        <v>00</v>
+        <v>FF</v>
       </c>
     </row>
     <row r="39" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB39" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC39" t="str">
-        <f t="shared" si="9"/>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(L10:L17)</f>
+        <v>00011000</v>
       </c>
       <c r="AD39" t="str">
         <f t="shared" si="4"/>
-        <v>00</v>
+        <v>18</v>
       </c>
     </row>
     <row r="40" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB40" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC40" t="str">
-        <f t="shared" si="9"/>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(K10:K17)</f>
+        <v>00011000</v>
       </c>
       <c r="AD40" t="str">
         <f t="shared" si="4"/>
-        <v>00</v>
+        <v>18</v>
       </c>
     </row>
     <row r="41" spans="28:30" x14ac:dyDescent="0.25">
       <c r="AB41" s="10" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="AC41" t="str">
-        <f t="shared" si="9"/>
-        <v>00000000</v>
+        <f>_xlfn.CONCAT(J10:J17)</f>
+        <v>00011000</v>
       </c>
       <c r="AD41" t="str">
         <f t="shared" si="4"/>
-        <v>00</v>
+        <v>18</v>
       </c>
     </row>
     <row r="42" spans="28:30" x14ac:dyDescent="0.25">
@@ -9095,5 +9050,6 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>